<commit_message>
Scinde les états financiers : un onglet par état et un onglet de contrôles
BILAN, COMPTE DE RESULTAT, TFT et CONTROLES remplacent l'onglet unique.
Ajoute les contrôles de variation des capitaux propres et de trésorerie
d'ouverture, avec une synthèse du nombre d'anomalies.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017qsfV16W64D6M2WCay1xb5
</commit_message>
<xml_diff>
--- a/previsions/PREVISIONS_FINANCIERES_5ANS_SYSCOHADA.xlsx
+++ b/previsions/PREVISIONS_FINANCIERES_5ANS_SYSCOHADA.xlsx
@@ -10,7 +10,10 @@
   <sheets>
     <sheet name="HYPOTHESES" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="BALANCES" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="ETATS FINANCIERS" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="BILAN" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="COMPTE DE RESULTAT" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="TFT" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="CONTROLES" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -44,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="506">
   <si>
     <t xml:space="preserve">PRÉVISIONS FINANCIÈRES SUR 5 ANS : HYPOTHÈSES</t>
   </si>
@@ -835,10 +838,10 @@
     <t xml:space="preserve">Règles de projection : capitaux, emprunts, immobilisations et amortissements depuis HYPOTHESES (sections 3-4) ; clients et fournisseurs selon les délais ; dettes sociales et fiscales proportionnelles aux charges 66 et 64 ; charges de détail réparties selon leur poids dans la balance de base ; la banque est le solde de trésorerie qui équilibre la balance (si négative, elle passe au crédit = concours bancaire DR).</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNTHÈSE DES ÉTATS FINANCIERS SUR 5 ANS (modèle SYSCOHADA révisé, système normal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bilan, compte de résultat et tableau des flux de trésorerie alimentés par les balances. Montants en FCFA.</t>
+    <t xml:space="preserve">BILAN PRÉVISIONNEL SUR 5 ANS (modèle SYSCOHADA révisé, système normal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimenté par l'onglet BALANCES. Valeurs nettes d'amortissements et de dépréciations. Montants en FCFA.</t>
   </si>
   <si>
     <t xml:space="preserve">Réf.</t>
@@ -1117,6 +1120,12 @@
     <t xml:space="preserve">TOTAL GÉNÉRAL PASSIF</t>
   </si>
   <si>
+    <t xml:space="preserve">COMPTE DE RÉSULTAT PRÉVISIONNEL SUR 5 ANS (modèle SYSCOHADA révisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimenté par l'onglet BALANCES. Charges présentées en négatif, soldes intermédiaires XA à XI. Montants en FCFA.</t>
+  </si>
+  <si>
     <t xml:space="preserve">COMPTE DE RÉSULTAT (charges en négatif)</t>
   </si>
   <si>
@@ -1321,6 +1330,12 @@
     <t xml:space="preserve">RÉSULTAT NET</t>
   </si>
   <si>
+    <t xml:space="preserve">TABLEAU DES FLUX DE TRÉSORERIE PRÉVISIONNEL SUR 5 ANS (modèle SYSCOHADA révisé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Méthode indirecte à partir de la CAFG, calculé par différence entre bilans successifs. Montants en FCFA.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TABLEAU DES FLUX DE TRÉSORERIE</t>
   </si>
   <si>
@@ -1480,6 +1495,45 @@
     <t xml:space="preserve">TFT de l'année de base non calculé : il nécessite le bilan de l'exercice précédent.</t>
   </si>
   <si>
+    <t xml:space="preserve">CONTRÔLES DE COHÉRENCE ET INDICATEURS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérifications croisées balances / bilan / compte de résultat / TFT. Toute valeur différente de 0 signale une anomalie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTRÔLES DE COHÉRENCE (tous doivent afficher 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance équilibrée : total débits - total crédits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilan équilibré : BZ - DZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat : XI du compte de résultat - résultat calculé (HYPOTHESES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TFT : ZH - (BT - DT) du bilan de clôture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capitaux propres : CP - (CP N-1 + XI - dividendes + apports + subventions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trésorerie d'ouverture : ZA - trésorerie nette de clôture N-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerte : trésorerie nette négative (1 = oui)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerte : capitaux propres &lt; moitié du capital (AUSCGIE art. 664)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthèse : nombre d'anomalies et d'alertes</t>
+  </si>
+  <si>
     <t xml:space="preserve">INDICATEURS DE GESTION</t>
   </si>
   <si>
@@ -1511,27 +1565,6 @@
   </si>
   <si>
     <t xml:space="preserve">Rentabilité des capitaux propres (XI / CP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONTRÔLES DE COHÉRENCE (tous doivent afficher 0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balance équilibrée : total débits - total crédits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bilan équilibré : BZ - DZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résultat : XI du compte de résultat - résultat calculé (HYPOTHESES)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TFT : ZH - (BT - DT) du bilan de clôture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alerte : trésorerie nette négative (1 = oui)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alerte : capitaux propres &lt; moitié du capital (AUSCGIE art. 664)</t>
   </si>
 </sst>
 </file>
@@ -1673,7 +1706,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1701,13 +1734,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1752,7 +1791,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1921,6 +1960,14 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1978,7 +2025,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -9116,7 +9163,7 @@
     <tabColor rgb="FF70AD47"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I152"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -9136,6 +9183,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -10265,28 +10313,28 @@
       <c r="B40" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="C40" s="18" t="n">
-        <f aca="false">C104</f>
+      <c r="C40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!C47</f>
         <v>72698877</v>
       </c>
-      <c r="D40" s="18" t="n">
-        <f aca="false">D104</f>
+      <c r="D40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!D47</f>
         <v>69668558.94115</v>
       </c>
-      <c r="E40" s="18" t="n">
-        <f aca="false">E104</f>
+      <c r="E40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!E47</f>
         <v>73449452.3537075</v>
       </c>
-      <c r="F40" s="18" t="n">
-        <f aca="false">F104</f>
+      <c r="F40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!F47</f>
         <v>80232556.3043929</v>
       </c>
-      <c r="G40" s="18" t="n">
-        <f aca="false">G104</f>
+      <c r="G40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!G47</f>
         <v>88085549.0071126</v>
       </c>
-      <c r="H40" s="18" t="n">
-        <f aca="false">H104</f>
+      <c r="H40" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!H47</f>
         <v>102613790.444968</v>
       </c>
     </row>
@@ -10942,2779 +10990,3029 @@
         <v>0.0459796911793886</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="36" t="s">
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF70AD47"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:I47"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="str">
+        <f aca="false">"Entité : "&amp;HYPOTHESES!$C$4</f>
+        <v>Entité : MON ENTREPRISE</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="36" t="s">
         <v>265</v>
       </c>
-      <c r="B62" s="36" t="s">
-        <v>357</v>
-      </c>
-      <c r="C62" s="36" t="str">
+      <c r="B5" s="36" t="s">
+        <v>359</v>
+      </c>
+      <c r="C5" s="36" t="str">
         <f aca="false">"Réel "&amp;HYPOTHESES!$C$5</f>
         <v>Réel 2024</v>
       </c>
-      <c r="D62" s="37" t="n">
+      <c r="D5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+1</f>
         <v>2025</v>
       </c>
-      <c r="E62" s="37" t="n">
+      <c r="E5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+2</f>
         <v>2026</v>
       </c>
-      <c r="F62" s="37" t="n">
+      <c r="F5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+3</f>
         <v>2027</v>
       </c>
-      <c r="G62" s="37" t="n">
+      <c r="G5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+4</f>
         <v>2028</v>
       </c>
-      <c r="H62" s="37" t="n">
+      <c r="H5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+5</f>
         <v>2029</v>
       </c>
-      <c r="I62" s="36" t="s">
+      <c r="I5" s="36" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="13" t="s">
-        <v>358</v>
-      </c>
-      <c r="B63" s="12" t="s">
-        <v>359</v>
-      </c>
-      <c r="C63" s="15" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="C6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
-      <c r="D63" s="15" t="n">
+      <c r="D6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
-      <c r="E63" s="15" t="n">
+      <c r="E6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
-      <c r="F63" s="15" t="n">
+      <c r="F6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
-      <c r="G63" s="15" t="n">
+      <c r="G6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
-      <c r="H63" s="15" t="n">
+      <c r="H6" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TA")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TA"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="B64" s="12" t="s">
-        <v>361</v>
-      </c>
-      <c r="C64" s="15" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>362</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="C7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
-      <c r="D64" s="15" t="n">
+      <c r="D7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
-      <c r="E64" s="15" t="n">
+      <c r="E7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
-      <c r="F64" s="15" t="n">
+      <c r="F7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
-      <c r="G64" s="15" t="n">
+      <c r="G7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
-      <c r="H64" s="15" t="n">
+      <c r="H7" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RA")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RA"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="13" t="s">
-        <v>362</v>
-      </c>
-      <c r="B65" s="12" t="s">
-        <v>363</v>
-      </c>
-      <c r="C65" s="15" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="C8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
-      <c r="D65" s="15" t="n">
+      <c r="D8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
-      <c r="E65" s="15" t="n">
+      <c r="E8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
-      <c r="F65" s="15" t="n">
+      <c r="F8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
-      <c r="G65" s="15" t="n">
+      <c r="G8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
-      <c r="H65" s="15" t="n">
+      <c r="H8" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RB")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RB"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="34" t="s">
-        <v>364</v>
-      </c>
-      <c r="B66" s="34" t="s">
-        <v>365</v>
-      </c>
-      <c r="C66" s="35" t="n">
-        <f aca="false">C63+C64+C65</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="35" t="n">
-        <f aca="false">D63+D64+D65</f>
-        <v>0</v>
-      </c>
-      <c r="E66" s="35" t="n">
-        <f aca="false">E63+E64+E65</f>
-        <v>0</v>
-      </c>
-      <c r="F66" s="35" t="n">
-        <f aca="false">F63+F64+F65</f>
-        <v>0</v>
-      </c>
-      <c r="G66" s="35" t="n">
-        <f aca="false">G63+G64+G65</f>
-        <v>0</v>
-      </c>
-      <c r="H66" s="35" t="n">
-        <f aca="false">H63+H64+H65</f>
-        <v>0</v>
-      </c>
-      <c r="I66" s="38"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="13" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="34" t="s">
         <v>366</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B9" s="34" t="s">
         <v>367</v>
       </c>
-      <c r="C67" s="15" t="n">
+      <c r="C9" s="35" t="n">
+        <f aca="false">C6+C7+C8</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <f aca="false">D6+D7+D8</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <f aca="false">E6+E7+E8</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="35" t="n">
+        <f aca="false">F6+F7+F8</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <f aca="false">G6+G7+G8</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <f aca="false">H6+H7+H8</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="38"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="C10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
-      <c r="D67" s="15" t="n">
+      <c r="D10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
-      <c r="E67" s="15" t="n">
+      <c r="E10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
-      <c r="F67" s="15" t="n">
+      <c r="F10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
-      <c r="G67" s="15" t="n">
+      <c r="G10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
-      <c r="H67" s="15" t="n">
+      <c r="H10" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TB")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TB"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="13" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="B68" s="12" t="s">
-        <v>368</v>
-      </c>
-      <c r="C68" s="15" t="n">
+      <c r="B11" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="C11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TC"))</f>
         <v>701026695</v>
       </c>
-      <c r="D68" s="15" t="n">
+      <c r="D11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TC"))</f>
         <v>736078029.75</v>
       </c>
-      <c r="E68" s="15" t="n">
+      <c r="E11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TC"))</f>
         <v>772881931.2375</v>
       </c>
-      <c r="F68" s="15" t="n">
+      <c r="F11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TC"))</f>
         <v>811526027.799375</v>
       </c>
-      <c r="G68" s="15" t="n">
+      <c r="G11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TC"))</f>
         <v>852102329.189344</v>
       </c>
-      <c r="H68" s="15" t="n">
+      <c r="H11" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TC")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TC"))</f>
         <v>894707445.648811</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="13" t="s">
-        <v>369</v>
-      </c>
-      <c r="B69" s="12" t="s">
-        <v>370</v>
-      </c>
-      <c r="C69" s="15" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="C12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
-      <c r="D69" s="15" t="n">
+      <c r="D12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
-      <c r="E69" s="15" t="n">
+      <c r="E12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
-      <c r="F69" s="15" t="n">
+      <c r="F12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
-      <c r="G69" s="15" t="n">
+      <c r="G12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
-      <c r="H69" s="15" t="n">
+      <c r="H12" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TD")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TD"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="34" t="s">
-        <v>371</v>
-      </c>
-      <c r="B70" s="34" t="s">
-        <v>372</v>
-      </c>
-      <c r="C70" s="35" t="n">
-        <f aca="false">C63+C67+C68+C69</f>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="34" t="s">
+        <v>373</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>374</v>
+      </c>
+      <c r="C13" s="35" t="n">
+        <f aca="false">C6+C10+C11+C12</f>
         <v>701026695</v>
       </c>
-      <c r="D70" s="35" t="n">
-        <f aca="false">D63+D67+D68+D69</f>
+      <c r="D13" s="35" t="n">
+        <f aca="false">D6+D10+D11+D12</f>
         <v>736078029.75</v>
       </c>
-      <c r="E70" s="35" t="n">
-        <f aca="false">E63+E67+E68+E69</f>
+      <c r="E13" s="35" t="n">
+        <f aca="false">E6+E10+E11+E12</f>
         <v>772881931.2375</v>
       </c>
-      <c r="F70" s="35" t="n">
-        <f aca="false">F63+F67+F68+F69</f>
+      <c r="F13" s="35" t="n">
+        <f aca="false">F6+F10+F11+F12</f>
         <v>811526027.799375</v>
       </c>
-      <c r="G70" s="35" t="n">
-        <f aca="false">G63+G67+G68+G69</f>
+      <c r="G13" s="35" t="n">
+        <f aca="false">G6+G10+G11+G12</f>
         <v>852102329.189344</v>
       </c>
-      <c r="H70" s="35" t="n">
-        <f aca="false">H63+H67+H68+H69</f>
+      <c r="H13" s="35" t="n">
+        <f aca="false">H6+H10+H11+H12</f>
         <v>894707445.648811</v>
       </c>
-      <c r="I70" s="39" t="n">
-        <f aca="false">IF(OR(C70&lt;=0,H70&lt;=0),"",(H70/C70)^(1/5)-1)</f>
+      <c r="I13" s="39" t="n">
+        <f aca="false">IF(OR(C13&lt;=0,H13&lt;=0),"",(H13/C13)^(1/5)-1)</f>
         <v>0.05</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="13" t="s">
-        <v>373</v>
-      </c>
-      <c r="B71" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="C71" s="15" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="C14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
-      <c r="D71" s="15" t="n">
+      <c r="D14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
-      <c r="E71" s="15" t="n">
+      <c r="E14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
-      <c r="F71" s="15" t="n">
+      <c r="F14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
-      <c r="G71" s="15" t="n">
+      <c r="G14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
-      <c r="H71" s="15" t="n">
+      <c r="H14" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TE")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TE"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="13" t="s">
-        <v>375</v>
-      </c>
-      <c r="B72" s="12" t="s">
-        <v>376</v>
-      </c>
-      <c r="C72" s="15" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="C15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
-      <c r="D72" s="15" t="n">
+      <c r="D15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
-      <c r="E72" s="15" t="n">
+      <c r="E15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
-      <c r="F72" s="15" t="n">
+      <c r="F15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
-      <c r="G72" s="15" t="n">
+      <c r="G15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
-      <c r="H72" s="15" t="n">
+      <c r="H15" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TF")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TF"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="13" t="s">
-        <v>377</v>
-      </c>
-      <c r="B73" s="12" t="s">
-        <v>378</v>
-      </c>
-      <c r="C73" s="15" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="C16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
-      <c r="D73" s="15" t="n">
+      <c r="D16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
-      <c r="E73" s="15" t="n">
+      <c r="E16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
-      <c r="F73" s="15" t="n">
+      <c r="F16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
-      <c r="G73" s="15" t="n">
+      <c r="G16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
-      <c r="H73" s="15" t="n">
+      <c r="H16" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TG")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TG"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="B74" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="C74" s="15" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="C17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
-      <c r="D74" s="15" t="n">
+      <c r="D17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
-      <c r="E74" s="15" t="n">
+      <c r="E17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
-      <c r="F74" s="15" t="n">
+      <c r="F17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
-      <c r="G74" s="15" t="n">
+      <c r="G17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
-      <c r="H74" s="15" t="n">
+      <c r="H17" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TH")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TH"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="B75" s="12" t="s">
-        <v>382</v>
-      </c>
-      <c r="C75" s="15" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>383</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="C18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
-      <c r="D75" s="15" t="n">
+      <c r="D18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
-      <c r="E75" s="15" t="n">
+      <c r="E18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
-      <c r="F75" s="15" t="n">
+      <c r="F18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
-      <c r="G75" s="15" t="n">
+      <c r="G18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
-      <c r="H75" s="15" t="n">
+      <c r="H18" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TI")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TI"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="13" t="s">
-        <v>383</v>
-      </c>
-      <c r="B76" s="12" t="s">
-        <v>384</v>
-      </c>
-      <c r="C76" s="15" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="C19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
-      <c r="D76" s="15" t="n">
+      <c r="D19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
-      <c r="E76" s="15" t="n">
+      <c r="E19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
-      <c r="F76" s="15" t="n">
+      <c r="F19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
-      <c r="G76" s="15" t="n">
+      <c r="G19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
-      <c r="H76" s="15" t="n">
+      <c r="H19" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RC")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RC"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="13" t="s">
-        <v>385</v>
-      </c>
-      <c r="B77" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="C77" s="15" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="C20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
-      <c r="D77" s="15" t="n">
+      <c r="D20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
-      <c r="E77" s="15" t="n">
+      <c r="E20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
-      <c r="F77" s="15" t="n">
+      <c r="F20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
-      <c r="G77" s="15" t="n">
+      <c r="G20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
-      <c r="H77" s="15" t="n">
+      <c r="H20" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RD")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RD"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="13" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="B78" s="12" t="s">
-        <v>387</v>
-      </c>
-      <c r="C78" s="15" t="n">
+      <c r="B21" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="C21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RE"))</f>
         <v>-278141464</v>
       </c>
-      <c r="D78" s="15" t="n">
+      <c r="D21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RE"))</f>
         <v>-292075762.2048</v>
       </c>
-      <c r="E78" s="15" t="n">
+      <c r="E21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RE"))</f>
         <v>-306679550.31504</v>
       </c>
-      <c r="F78" s="15" t="n">
+      <c r="F21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RE"))</f>
         <v>-322013527.830792</v>
       </c>
-      <c r="G78" s="15" t="n">
+      <c r="G21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RE"))</f>
         <v>-338114204.222332</v>
       </c>
-      <c r="H78" s="15" t="n">
+      <c r="H21" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RE")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RE"))</f>
         <v>-355019914.433448</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="13" t="s">
-        <v>388</v>
-      </c>
-      <c r="B79" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="C79" s="15" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="C22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
-      <c r="D79" s="15" t="n">
+      <c r="D22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
-      <c r="E79" s="15" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
-      <c r="F79" s="15" t="n">
+      <c r="F22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
-      <c r="G79" s="15" t="n">
+      <c r="G22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
-      <c r="H79" s="15" t="n">
+      <c r="H22" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RF")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RF"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="13" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B23" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C80" s="15" t="n">
+      <c r="C23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RG"))</f>
         <v>-3820098</v>
       </c>
-      <c r="D80" s="15" t="n">
+      <c r="D23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RG"))</f>
         <v>-3974821.36065</v>
       </c>
-      <c r="E80" s="15" t="n">
+      <c r="E23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RG"))</f>
         <v>-4173562.4286825</v>
       </c>
-      <c r="F80" s="15" t="n">
+      <c r="F23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RG"))</f>
         <v>-4382240.55011663</v>
       </c>
-      <c r="G80" s="15" t="n">
+      <c r="G23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RG"))</f>
         <v>-4601352.57762246</v>
       </c>
-      <c r="H80" s="15" t="n">
+      <c r="H23" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RG")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RG"))</f>
         <v>-4831420.20650358</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="13" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B24" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C81" s="15" t="n">
+      <c r="C24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RH"))</f>
         <v>-106769083</v>
       </c>
-      <c r="D81" s="15" t="n">
+      <c r="D24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RH"))</f>
         <v>-112104683.930925</v>
       </c>
-      <c r="E81" s="15" t="n">
+      <c r="E24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RH"))</f>
         <v>-117709918.127471</v>
       </c>
-      <c r="F81" s="15" t="n">
+      <c r="F24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RH"))</f>
         <v>-123595414.033845</v>
       </c>
-      <c r="G81" s="15" t="n">
+      <c r="G24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RH"))</f>
         <v>-129775184.735537</v>
       </c>
-      <c r="H81" s="15" t="n">
+      <c r="H24" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RH")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RH"))</f>
         <v>-136263943.972314</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="13" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B25" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C82" s="15" t="n">
+      <c r="C25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RI"))</f>
         <v>-14869670</v>
       </c>
-      <c r="D82" s="15" t="n">
+      <c r="D25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RI"))</f>
         <v>-15604854.2307</v>
       </c>
-      <c r="E82" s="15" t="n">
+      <c r="E25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RI"))</f>
         <v>-16385096.942235</v>
       </c>
-      <c r="F82" s="15" t="n">
+      <c r="F25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RI"))</f>
         <v>-17204351.7893468</v>
       </c>
-      <c r="G82" s="15" t="n">
+      <c r="G25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RI"))</f>
         <v>-18064569.3788141</v>
       </c>
-      <c r="H82" s="15" t="n">
+      <c r="H25" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RI")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RI"))</f>
         <v>-18967797.8477548</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="13" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B26" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C83" s="15" t="n">
+      <c r="C26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RJ"))</f>
         <v>-1316731</v>
       </c>
-      <c r="D83" s="15" t="n">
+      <c r="D26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RJ"))</f>
         <v>-1398548.256525</v>
       </c>
-      <c r="E83" s="15" t="n">
+      <c r="E26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RJ"))</f>
         <v>-1468475.66935125</v>
       </c>
-      <c r="F83" s="15" t="n">
+      <c r="F26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RJ"))</f>
         <v>-1541899.45281881</v>
       </c>
-      <c r="G83" s="15" t="n">
+      <c r="G26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RJ"))</f>
         <v>-1618994.42545975</v>
       </c>
-      <c r="H83" s="15" t="n">
+      <c r="H26" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RJ")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RJ"))</f>
         <v>-1699944.14673274</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="34" t="s">
-        <v>390</v>
-      </c>
-      <c r="B84" s="34" t="s">
-        <v>391</v>
-      </c>
-      <c r="C84" s="35" t="n">
-        <f aca="false">C70+C64+C65+C71+C72+C73+C74+C75+C76+C77+C78+C79+C80+C81+C82+C83</f>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="34" t="s">
+        <v>392</v>
+      </c>
+      <c r="B27" s="34" t="s">
+        <v>393</v>
+      </c>
+      <c r="C27" s="35" t="n">
+        <f aca="false">C13+C7+C8+C14+C15+C16+C17+C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
         <v>296109649</v>
       </c>
-      <c r="D84" s="35" t="n">
-        <f aca="false">D70+D64+D65+D71+D72+D73+D74+D75+D76+D77+D78+D79+D80+D81+D82+D83</f>
+      <c r="D27" s="35" t="n">
+        <f aca="false">D13+D7+D8+D14+D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
         <v>310919359.7664</v>
       </c>
-      <c r="E84" s="35" t="n">
-        <f aca="false">E70+E64+E65+E71+E72+E73+E74+E75+E76+E77+E78+E79+E80+E81+E82+E83</f>
+      <c r="E27" s="35" t="n">
+        <f aca="false">E13+E7+E8+E14+E15+E16+E17+E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
         <v>326465327.75472</v>
       </c>
-      <c r="F84" s="35" t="n">
-        <f aca="false">F70+F64+F65+F71+F72+F73+F74+F75+F76+F77+F78+F79+F80+F81+F82+F83</f>
+      <c r="F27" s="35" t="n">
+        <f aca="false">F13+F7+F8+F14+F15+F16+F17+F18+F19+F20+F21+F22+F23+F24+F25+F26</f>
         <v>342788594.142456</v>
       </c>
-      <c r="G84" s="35" t="n">
-        <f aca="false">G70+G64+G65+G71+G72+G73+G74+G75+G76+G77+G78+G79+G80+G81+G82+G83</f>
+      <c r="G27" s="35" t="n">
+        <f aca="false">G13+G7+G8+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G24+G25+G26</f>
         <v>359928023.849579</v>
       </c>
-      <c r="H84" s="35" t="n">
-        <f aca="false">H70+H64+H65+H71+H72+H73+H74+H75+H76+H77+H78+H79+H80+H81+H82+H83</f>
+      <c r="H27" s="35" t="n">
+        <f aca="false">H13+H7+H8+H14+H15+H16+H17+H18+H19+H20+H21+H22+H23+H24+H25+H26</f>
         <v>377924425.042058</v>
       </c>
-      <c r="I84" s="38"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="13" t="s">
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B28" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C85" s="15" t="n">
+      <c r="C28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RK"))</f>
         <v>-106025515</v>
       </c>
-      <c r="D85" s="15" t="n">
+      <c r="D28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RK"))</f>
         <v>-111294998.0982</v>
       </c>
-      <c r="E85" s="15" t="n">
+      <c r="E28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RK"))</f>
         <v>-116859748.00311</v>
       </c>
-      <c r="F85" s="15" t="n">
+      <c r="F28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RK"))</f>
         <v>-122702735.403266</v>
       </c>
-      <c r="G85" s="15" t="n">
+      <c r="G28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RK"))</f>
         <v>-128837872.173429</v>
       </c>
-      <c r="H85" s="15" t="n">
+      <c r="H28" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RK")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RK"))</f>
         <v>-135279765.7821</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="34" t="s">
-        <v>392</v>
-      </c>
-      <c r="B86" s="34" t="s">
-        <v>393</v>
-      </c>
-      <c r="C86" s="35" t="n">
-        <f aca="false">C84+C85</f>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="34" t="s">
+        <v>394</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>395</v>
+      </c>
+      <c r="C29" s="35" t="n">
+        <f aca="false">C27+C28</f>
         <v>190084134</v>
       </c>
-      <c r="D86" s="35" t="n">
-        <f aca="false">D84+D85</f>
+      <c r="D29" s="35" t="n">
+        <f aca="false">D27+D28</f>
         <v>199624361.6682</v>
       </c>
-      <c r="E86" s="35" t="n">
-        <f aca="false">E84+E85</f>
+      <c r="E29" s="35" t="n">
+        <f aca="false">E27+E28</f>
         <v>209605579.75161</v>
       </c>
-      <c r="F86" s="35" t="n">
-        <f aca="false">F84+F85</f>
+      <c r="F29" s="35" t="n">
+        <f aca="false">F27+F28</f>
         <v>220085858.739191</v>
       </c>
-      <c r="G86" s="35" t="n">
-        <f aca="false">G84+G85</f>
+      <c r="G29" s="35" t="n">
+        <f aca="false">G27+G28</f>
         <v>231090151.67615</v>
       </c>
-      <c r="H86" s="35" t="n">
-        <f aca="false">H84+H85</f>
+      <c r="H29" s="35" t="n">
+        <f aca="false">H27+H28</f>
         <v>242644659.259958</v>
       </c>
-      <c r="I86" s="39" t="n">
-        <f aca="false">IF(OR(C86&lt;=0,H86&lt;=0),"",(H86/C86)^(1/5)-1)</f>
+      <c r="I29" s="39" t="n">
+        <f aca="false">IF(OR(C29&lt;=0,H29&lt;=0),"",(H29/C29)^(1/5)-1)</f>
         <v>0.0500378972903746</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="13" t="s">
-        <v>394</v>
-      </c>
-      <c r="B87" s="12" t="s">
-        <v>395</v>
-      </c>
-      <c r="C87" s="15" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="C30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
-      <c r="D87" s="15" t="n">
+      <c r="D30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
-      <c r="E87" s="15" t="n">
+      <c r="E30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
-      <c r="F87" s="15" t="n">
+      <c r="F30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
-      <c r="G87" s="15" t="n">
+      <c r="G30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
-      <c r="H87" s="15" t="n">
+      <c r="H30" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TJ")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TJ"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="13" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="B88" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="C88" s="15" t="n">
+      <c r="B31" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="C31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RL"))</f>
         <v>-85892595</v>
       </c>
-      <c r="D88" s="15" t="n">
+      <c r="D31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RL"))</f>
         <v>-103559261.666667</v>
       </c>
-      <c r="E88" s="15" t="n">
+      <c r="E31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RL"))</f>
         <v>-110935217.333333</v>
       </c>
-      <c r="F88" s="15" t="n">
+      <c r="F31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RL"))</f>
         <v>-113957711</v>
       </c>
-      <c r="G88" s="15" t="n">
+      <c r="G31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RL"))</f>
         <v>-114491347</v>
       </c>
-      <c r="H88" s="15" t="n">
+      <c r="H31" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RL")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RL"))</f>
         <v>-106674866</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="34" t="s">
-        <v>397</v>
-      </c>
-      <c r="B89" s="34" t="s">
-        <v>398</v>
-      </c>
-      <c r="C89" s="35" t="n">
-        <f aca="false">C86+C87+C88</f>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="34" t="s">
+        <v>399</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>400</v>
+      </c>
+      <c r="C32" s="35" t="n">
+        <f aca="false">C29+C30+C31</f>
         <v>104191539</v>
       </c>
-      <c r="D89" s="35" t="n">
-        <f aca="false">D86+D87+D88</f>
+      <c r="D32" s="35" t="n">
+        <f aca="false">D29+D30+D31</f>
         <v>96065100.0015333</v>
       </c>
-      <c r="E89" s="35" t="n">
-        <f aca="false">E86+E87+E88</f>
+      <c r="E32" s="35" t="n">
+        <f aca="false">E29+E30+E31</f>
         <v>98670362.4182767</v>
       </c>
-      <c r="F89" s="35" t="n">
-        <f aca="false">F86+F87+F88</f>
+      <c r="F32" s="35" t="n">
+        <f aca="false">F29+F30+F31</f>
         <v>106128147.739191</v>
       </c>
-      <c r="G89" s="35" t="n">
-        <f aca="false">G86+G87+G88</f>
+      <c r="G32" s="35" t="n">
+        <f aca="false">G29+G30+G31</f>
         <v>116598804.67615</v>
       </c>
-      <c r="H89" s="35" t="n">
-        <f aca="false">H86+H87+H88</f>
+      <c r="H32" s="35" t="n">
+        <f aca="false">H29+H30+H31</f>
         <v>135969793.259958</v>
       </c>
-      <c r="I89" s="38"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="13" t="s">
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="B90" s="12" t="s">
-        <v>399</v>
-      </c>
-      <c r="C90" s="15" t="n">
+      <c r="B33" s="12" t="s">
+        <v>401</v>
+      </c>
+      <c r="C33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
-      <c r="D90" s="15" t="n">
+      <c r="D33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
-      <c r="E90" s="15" t="n">
+      <c r="E33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
-      <c r="F90" s="15" t="n">
+      <c r="F33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
-      <c r="G90" s="15" t="n">
+      <c r="G33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
-      <c r="H90" s="15" t="n">
+      <c r="H33" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TK")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TK"))</f>
         <v>848594</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="13" t="s">
-        <v>400</v>
-      </c>
-      <c r="B91" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="C91" s="15" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="C34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
-      <c r="D91" s="15" t="n">
+      <c r="D34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
-      <c r="E91" s="15" t="n">
+      <c r="E34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
-      <c r="F91" s="15" t="n">
+      <c r="F34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
-      <c r="G91" s="15" t="n">
+      <c r="G34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
-      <c r="H91" s="15" t="n">
+      <c r="H34" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TL")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TL"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="13" t="s">
-        <v>402</v>
-      </c>
-      <c r="B92" s="12" t="s">
-        <v>403</v>
-      </c>
-      <c r="C92" s="15" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="C35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
-      <c r="D92" s="15" t="n">
+      <c r="D35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
-      <c r="E92" s="15" t="n">
+      <c r="E35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
-      <c r="F92" s="15" t="n">
+      <c r="F35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
-      <c r="G92" s="15" t="n">
+      <c r="G35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
-      <c r="H92" s="15" t="n">
+      <c r="H35" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TM")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TM"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="13" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
         <v>245</v>
       </c>
-      <c r="B93" s="12" t="s">
-        <v>404</v>
-      </c>
-      <c r="C93" s="15" t="n">
+      <c r="B36" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="C36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RM"))</f>
         <v>-8108297</v>
       </c>
-      <c r="D93" s="15" t="n">
+      <c r="D36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RM"))</f>
         <v>-4022282.08</v>
       </c>
-      <c r="E93" s="15" t="n">
+      <c r="E36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RM"))</f>
         <v>-1586353.28</v>
       </c>
-      <c r="F93" s="15" t="n">
+      <c r="F36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RM"))</f>
         <v>0</v>
       </c>
-      <c r="G93" s="15" t="n">
+      <c r="G36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RM"))</f>
         <v>0</v>
       </c>
-      <c r="H93" s="15" t="n">
+      <c r="H36" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RM")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RM"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="B94" s="12" t="s">
-        <v>406</v>
-      </c>
-      <c r="C94" s="15" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="C37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
-      <c r="D94" s="15" t="n">
+      <c r="D37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
-      <c r="E94" s="15" t="n">
+      <c r="E37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
-      <c r="F94" s="15" t="n">
+      <c r="F37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
-      <c r="G94" s="15" t="n">
+      <c r="G37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
-      <c r="H94" s="15" t="n">
+      <c r="H37" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RN")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RN"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="34" t="s">
-        <v>407</v>
-      </c>
-      <c r="B95" s="34" t="s">
-        <v>408</v>
-      </c>
-      <c r="C95" s="35" t="n">
-        <f aca="false">C90+C91+C92+C93+C94</f>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="34" t="s">
+        <v>409</v>
+      </c>
+      <c r="B38" s="34" t="s">
+        <v>410</v>
+      </c>
+      <c r="C38" s="35" t="n">
+        <f aca="false">C33+C34+C35+C36+C37</f>
         <v>-7259703</v>
       </c>
-      <c r="D95" s="35" t="n">
-        <f aca="false">D90+D91+D92+D93+D94</f>
+      <c r="D38" s="35" t="n">
+        <f aca="false">D33+D34+D35+D36+D37</f>
         <v>-3173688.08</v>
       </c>
-      <c r="E95" s="35" t="n">
-        <f aca="false">E90+E91+E92+E93+E94</f>
+      <c r="E38" s="35" t="n">
+        <f aca="false">E33+E34+E35+E36+E37</f>
         <v>-737759.28</v>
       </c>
-      <c r="F95" s="35" t="n">
-        <f aca="false">F90+F91+F92+F93+F94</f>
+      <c r="F38" s="35" t="n">
+        <f aca="false">F33+F34+F35+F36+F37</f>
         <v>848594</v>
       </c>
-      <c r="G95" s="35" t="n">
-        <f aca="false">G90+G91+G92+G93+G94</f>
+      <c r="G38" s="35" t="n">
+        <f aca="false">G33+G34+G35+G36+G37</f>
         <v>848594</v>
       </c>
-      <c r="H95" s="35" t="n">
-        <f aca="false">H90+H91+H92+H93+H94</f>
+      <c r="H38" s="35" t="n">
+        <f aca="false">H33+H34+H35+H36+H37</f>
         <v>848594</v>
       </c>
-      <c r="I95" s="38"/>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="34" t="s">
-        <v>409</v>
-      </c>
-      <c r="B96" s="34" t="s">
-        <v>410</v>
-      </c>
-      <c r="C96" s="35" t="n">
-        <f aca="false">C89+C95</f>
+      <c r="I38" s="38"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="34" t="s">
+        <v>411</v>
+      </c>
+      <c r="B39" s="34" t="s">
+        <v>412</v>
+      </c>
+      <c r="C39" s="35" t="n">
+        <f aca="false">C32+C38</f>
         <v>96931836</v>
       </c>
-      <c r="D96" s="35" t="n">
-        <f aca="false">D89+D95</f>
+      <c r="D39" s="35" t="n">
+        <f aca="false">D32+D38</f>
         <v>92891411.9215333</v>
       </c>
-      <c r="E96" s="35" t="n">
-        <f aca="false">E89+E95</f>
+      <c r="E39" s="35" t="n">
+        <f aca="false">E32+E38</f>
         <v>97932603.1382767</v>
       </c>
-      <c r="F96" s="35" t="n">
-        <f aca="false">F89+F95</f>
+      <c r="F39" s="35" t="n">
+        <f aca="false">F32+F38</f>
         <v>106976741.739191</v>
       </c>
-      <c r="G96" s="35" t="n">
-        <f aca="false">G89+G95</f>
+      <c r="G39" s="35" t="n">
+        <f aca="false">G32+G38</f>
         <v>117447398.67615</v>
       </c>
-      <c r="H96" s="35" t="n">
-        <f aca="false">H89+H95</f>
+      <c r="H39" s="35" t="n">
+        <f aca="false">H32+H38</f>
         <v>136818387.259958</v>
       </c>
-      <c r="I96" s="38"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="13" t="s">
-        <v>411</v>
-      </c>
-      <c r="B97" s="12" t="s">
-        <v>412</v>
-      </c>
-      <c r="C97" s="15" t="n">
+      <c r="I39" s="38"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>414</v>
+      </c>
+      <c r="C40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
-      <c r="D97" s="15" t="n">
+      <c r="D40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
-      <c r="E97" s="15" t="n">
+      <c r="E40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
-      <c r="F97" s="15" t="n">
+      <c r="F40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
-      <c r="G97" s="15" t="n">
+      <c r="G40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
-      <c r="H97" s="15" t="n">
+      <c r="H40" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TN")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TN"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="13" t="s">
-        <v>413</v>
-      </c>
-      <c r="B98" s="12" t="s">
-        <v>414</v>
-      </c>
-      <c r="C98" s="15" t="n">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>416</v>
+      </c>
+      <c r="C41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
-      <c r="D98" s="15" t="n">
+      <c r="D41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
-      <c r="E98" s="15" t="n">
+      <c r="E41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
-      <c r="F98" s="15" t="n">
+      <c r="F41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
-      <c r="G98" s="15" t="n">
+      <c r="G41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
-      <c r="H98" s="15" t="n">
+      <c r="H41" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"TO")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"TO"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="13" t="s">
-        <v>415</v>
-      </c>
-      <c r="B99" s="12" t="s">
-        <v>416</v>
-      </c>
-      <c r="C99" s="15" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>417</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="C42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
-      <c r="D99" s="15" t="n">
+      <c r="D42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
-      <c r="E99" s="15" t="n">
+      <c r="E42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
-      <c r="F99" s="15" t="n">
+      <c r="F42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
-      <c r="G99" s="15" t="n">
+      <c r="G42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
-      <c r="H99" s="15" t="n">
+      <c r="H42" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RO")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RO"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="13" t="s">
-        <v>417</v>
-      </c>
-      <c r="B100" s="12" t="s">
-        <v>418</v>
-      </c>
-      <c r="C100" s="15" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>419</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>420</v>
+      </c>
+      <c r="C43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
-      <c r="D100" s="15" t="n">
+      <c r="D43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
-      <c r="E100" s="15" t="n">
+      <c r="E43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
-      <c r="F100" s="15" t="n">
+      <c r="F43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
-      <c r="G100" s="15" t="n">
+      <c r="G43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
-      <c r="H100" s="15" t="n">
+      <c r="H43" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RP")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RP"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="34" t="s">
-        <v>419</v>
-      </c>
-      <c r="B101" s="34" t="s">
-        <v>420</v>
-      </c>
-      <c r="C101" s="35" t="n">
-        <f aca="false">C97+C98+C99+C100</f>
-        <v>0</v>
-      </c>
-      <c r="D101" s="35" t="n">
-        <f aca="false">D97+D98+D99+D100</f>
-        <v>0</v>
-      </c>
-      <c r="E101" s="35" t="n">
-        <f aca="false">E97+E98+E99+E100</f>
-        <v>0</v>
-      </c>
-      <c r="F101" s="35" t="n">
-        <f aca="false">F97+F98+F99+F100</f>
-        <v>0</v>
-      </c>
-      <c r="G101" s="35" t="n">
-        <f aca="false">G97+G98+G99+G100</f>
-        <v>0</v>
-      </c>
-      <c r="H101" s="35" t="n">
-        <f aca="false">H97+H98+H99+H100</f>
-        <v>0</v>
-      </c>
-      <c r="I101" s="38"/>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="13" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="34" t="s">
         <v>421</v>
       </c>
-      <c r="B102" s="12" t="s">
+      <c r="B44" s="34" t="s">
         <v>422</v>
       </c>
-      <c r="C102" s="15" t="n">
+      <c r="C44" s="35" t="n">
+        <f aca="false">C40+C41+C42+C43</f>
+        <v>0</v>
+      </c>
+      <c r="D44" s="35" t="n">
+        <f aca="false">D40+D41+D42+D43</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="35" t="n">
+        <f aca="false">E40+E41+E42+E43</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="35" t="n">
+        <f aca="false">F40+F41+F42+F43</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="35" t="n">
+        <f aca="false">G40+G41+G42+G43</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="35" t="n">
+        <f aca="false">H40+H41+H42+H43</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="38"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>423</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>424</v>
+      </c>
+      <c r="C45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
-      <c r="D102" s="15" t="n">
+      <c r="D45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
-      <c r="E102" s="15" t="n">
+      <c r="E45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
-      <c r="F102" s="15" t="n">
+      <c r="F45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
-      <c r="G102" s="15" t="n">
+      <c r="G45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
-      <c r="H102" s="15" t="n">
+      <c r="H45" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RQ")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RQ"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="13" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="B103" s="12" t="s">
-        <v>423</v>
-      </c>
-      <c r="C103" s="15" t="n">
+      <c r="B46" s="12" t="s">
+        <v>425</v>
+      </c>
+      <c r="C46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$E:$E,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"RS"))</f>
         <v>-24232959</v>
       </c>
-      <c r="D103" s="15" t="n">
+      <c r="D46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$G:$G,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"RS"))</f>
         <v>-23222852.9803833</v>
       </c>
-      <c r="E103" s="15" t="n">
+      <c r="E46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$I:$I,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"RS"))</f>
         <v>-24483150.7845692</v>
       </c>
-      <c r="F103" s="15" t="n">
+      <c r="F46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$K:$K,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"RS"))</f>
         <v>-26744185.4347976</v>
       </c>
-      <c r="G103" s="15" t="n">
+      <c r="G46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$M:$M,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"RS"))</f>
         <v>-29361849.6690375</v>
       </c>
-      <c r="H103" s="15" t="n">
+      <c r="H46" s="15" t="n">
         <f aca="false">SUMIFS(BALANCES!$O:$O,BALANCES!$C:$C,"RS")-(SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"RS"))</f>
         <v>-34204596.8149894</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="34" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="B104" s="34" t="s">
-        <v>424</v>
-      </c>
-      <c r="C104" s="35" t="n">
-        <f aca="false">C96+C101+C102+C103</f>
+      <c r="B47" s="34" t="s">
+        <v>426</v>
+      </c>
+      <c r="C47" s="35" t="n">
+        <f aca="false">C39+C44+C45+C46</f>
         <v>72698877</v>
       </c>
-      <c r="D104" s="35" t="n">
-        <f aca="false">D96+D101+D102+D103</f>
+      <c r="D47" s="35" t="n">
+        <f aca="false">D39+D44+D45+D46</f>
         <v>69668558.94115</v>
       </c>
-      <c r="E104" s="35" t="n">
-        <f aca="false">E96+E101+E102+E103</f>
+      <c r="E47" s="35" t="n">
+        <f aca="false">E39+E44+E45+E46</f>
         <v>73449452.3537075</v>
       </c>
-      <c r="F104" s="35" t="n">
-        <f aca="false">F96+F101+F102+F103</f>
+      <c r="F47" s="35" t="n">
+        <f aca="false">F39+F44+F45+F46</f>
         <v>80232556.3043929</v>
       </c>
-      <c r="G104" s="35" t="n">
-        <f aca="false">G96+G101+G102+G103</f>
+      <c r="G47" s="35" t="n">
+        <f aca="false">G39+G44+G45+G46</f>
         <v>88085549.0071126</v>
       </c>
-      <c r="H104" s="35" t="n">
-        <f aca="false">H96+H101+H102+H103</f>
+      <c r="H47" s="35" t="n">
+        <f aca="false">H39+H44+H45+H46</f>
         <v>102613790.444968</v>
       </c>
-      <c r="I104" s="39" t="n">
-        <f aca="false">IF(OR(C104&lt;=0,H104&lt;=0),"",(H104/C104)^(1/5)-1)</f>
+      <c r="I47" s="39" t="n">
+        <f aca="false">IF(OR(C47&lt;=0,H47&lt;=0),"",(H47/C47)^(1/5)-1)</f>
         <v>0.0713604390279148</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="36" t="s">
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF70AD47"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="str">
+        <f aca="false">"Entité : "&amp;HYPOTHESES!$C$4</f>
+        <v>Entité : MON ENTREPRISE</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="36" t="s">
         <v>265</v>
       </c>
-      <c r="B106" s="36" t="s">
-        <v>425</v>
-      </c>
-      <c r="C106" s="36" t="str">
+      <c r="B5" s="36" t="s">
+        <v>429</v>
+      </c>
+      <c r="C5" s="36" t="str">
         <f aca="false">"Réel "&amp;HYPOTHESES!$C$5</f>
         <v>Réel 2024</v>
       </c>
-      <c r="D106" s="37" t="n">
+      <c r="D5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+1</f>
         <v>2025</v>
       </c>
-      <c r="E106" s="37" t="n">
+      <c r="E5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+2</f>
         <v>2026</v>
       </c>
-      <c r="F106" s="37" t="n">
+      <c r="F5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+3</f>
         <v>2027</v>
       </c>
-      <c r="G106" s="37" t="n">
+      <c r="G5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+4</f>
         <v>2028</v>
       </c>
-      <c r="H106" s="37" t="n">
+      <c r="H5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+5</f>
         <v>2029</v>
       </c>
-      <c r="I106" s="36" t="s">
+      <c r="I5" s="36" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="34" t="s">
-        <v>426</v>
-      </c>
-      <c r="B107" s="34" t="s">
-        <v>427</v>
-      </c>
-      <c r="C107" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D107" s="35" t="n">
-        <f aca="false">C28-C58</f>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="34" t="s">
+        <v>430</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>431</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D6" s="35" t="n">
+        <f aca="false">BILAN!C28-BILAN!C58</f>
         <v>128133958</v>
       </c>
-      <c r="E107" s="35" t="n">
-        <f aca="false">D28-D58</f>
+      <c r="E6" s="35" t="n">
+        <f aca="false">BILAN!D28-BILAN!D58</f>
         <v>46216154.2754206</v>
       </c>
-      <c r="F107" s="35" t="n">
-        <f aca="false">E28-E58</f>
+      <c r="F6" s="35" t="n">
+        <f aca="false">BILAN!E28-BILAN!E58</f>
         <v>161168943.701008</v>
       </c>
-      <c r="G107" s="35" t="n">
-        <f aca="false">F28-F58</f>
+      <c r="G6" s="35" t="n">
+        <f aca="false">BILAN!F28-BILAN!F58</f>
         <v>305964345.486709</v>
       </c>
-      <c r="H107" s="35" t="n">
-        <f aca="false">G28-G58</f>
+      <c r="H6" s="35" t="n">
+        <f aca="false">BILAN!G28-BILAN!G58</f>
         <v>418670210.550694</v>
       </c>
-      <c r="I107" s="38"/>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="B108" s="12" t="s">
-        <v>430</v>
-      </c>
-      <c r="C108" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D108" s="18" t="n">
-        <f aca="false">D104-D88-D94-D87-D91-D99-D97</f>
+      <c r="I6" s="38"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>433</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!D47-'COMPTE DE RESULTAT'!D31-'COMPTE DE RESULTAT'!D37-'COMPTE DE RESULTAT'!D30-'COMPTE DE RESULTAT'!D34-'COMPTE DE RESULTAT'!D42-'COMPTE DE RESULTAT'!D40</f>
         <v>173227820.607817</v>
       </c>
-      <c r="E108" s="18" t="n">
-        <f aca="false">E104-E88-E94-E87-E91-E99-E97</f>
+      <c r="E7" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!E47-'COMPTE DE RESULTAT'!E31-'COMPTE DE RESULTAT'!E37-'COMPTE DE RESULTAT'!E30-'COMPTE DE RESULTAT'!E34-'COMPTE DE RESULTAT'!E42-'COMPTE DE RESULTAT'!E40</f>
         <v>184384669.687041</v>
       </c>
-      <c r="F108" s="18" t="n">
-        <f aca="false">F104-F88-F94-F87-F91-F99-F97</f>
+      <c r="F7" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!F47-'COMPTE DE RESULTAT'!F31-'COMPTE DE RESULTAT'!F37-'COMPTE DE RESULTAT'!F30-'COMPTE DE RESULTAT'!F34-'COMPTE DE RESULTAT'!F42-'COMPTE DE RESULTAT'!F40</f>
         <v>194190267.304393</v>
       </c>
-      <c r="G108" s="18" t="n">
-        <f aca="false">G104-G88-G94-G87-G91-G99-G97</f>
+      <c r="G7" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!G47-'COMPTE DE RESULTAT'!G31-'COMPTE DE RESULTAT'!G37-'COMPTE DE RESULTAT'!G30-'COMPTE DE RESULTAT'!G34-'COMPTE DE RESULTAT'!G42-'COMPTE DE RESULTAT'!G40</f>
         <v>202576896.007113</v>
       </c>
-      <c r="H108" s="18" t="n">
-        <f aca="false">H104-H88-H94-H87-H91-H99-H97</f>
+      <c r="H7" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!H47-'COMPTE DE RESULTAT'!H31-'COMPTE DE RESULTAT'!H37-'COMPTE DE RESULTAT'!H30-'COMPTE DE RESULTAT'!H34-'COMPTE DE RESULTAT'!H42-'COMPTE DE RESULTAT'!H40</f>
         <v>209288656.444968</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="13" t="s">
-        <v>431</v>
-      </c>
-      <c r="B109" s="12" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>435</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>436</v>
+      </c>
+      <c r="C8" s="41" t="s">
         <v>432</v>
       </c>
-      <c r="C109" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D109" s="18" t="n">
-        <f aca="false">-(D18-C18)</f>
+      <c r="D8" s="18" t="n">
+        <f aca="false">-(BILAN!D18-BILAN!C18)</f>
         <v>-0</v>
       </c>
-      <c r="E109" s="18" t="n">
-        <f aca="false">-(E18-D18)</f>
+      <c r="E8" s="18" t="n">
+        <f aca="false">-(BILAN!E18-BILAN!D18)</f>
         <v>-0</v>
       </c>
-      <c r="F109" s="18" t="n">
-        <f aca="false">-(F18-E18)</f>
+      <c r="F8" s="18" t="n">
+        <f aca="false">-(BILAN!F18-BILAN!E18)</f>
         <v>-0</v>
       </c>
-      <c r="G109" s="18" t="n">
-        <f aca="false">-(G18-F18)</f>
+      <c r="G8" s="18" t="n">
+        <f aca="false">-(BILAN!G18-BILAN!F18)</f>
         <v>-0</v>
       </c>
-      <c r="H109" s="18" t="n">
-        <f aca="false">-(H18-G18)</f>
+      <c r="H8" s="18" t="n">
+        <f aca="false">-(BILAN!H18-BILAN!G18)</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="13" t="s">
-        <v>433</v>
-      </c>
-      <c r="B110" s="12" t="s">
-        <v>434</v>
-      </c>
-      <c r="C110" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D110" s="18" t="n">
-        <f aca="false">-(D19-C19)</f>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>437</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>438</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <f aca="false">-(BILAN!D19-BILAN!C19)</f>
         <v>-0</v>
       </c>
-      <c r="E110" s="18" t="n">
-        <f aca="false">-(E19-D19)</f>
+      <c r="E9" s="18" t="n">
+        <f aca="false">-(BILAN!E19-BILAN!D19)</f>
         <v>-0</v>
       </c>
-      <c r="F110" s="18" t="n">
-        <f aca="false">-(F19-E19)</f>
+      <c r="F9" s="18" t="n">
+        <f aca="false">-(BILAN!F19-BILAN!E19)</f>
         <v>-0</v>
       </c>
-      <c r="G110" s="18" t="n">
-        <f aca="false">-(G19-F19)</f>
+      <c r="G9" s="18" t="n">
+        <f aca="false">-(BILAN!G19-BILAN!F19)</f>
         <v>-0</v>
       </c>
-      <c r="H110" s="18" t="n">
-        <f aca="false">-(H19-G19)</f>
+      <c r="H9" s="18" t="n">
+        <f aca="false">-(BILAN!H19-BILAN!G19)</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="13" t="s">
-        <v>435</v>
-      </c>
-      <c r="B111" s="12" t="s">
-        <v>436</v>
-      </c>
-      <c r="C111" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D111" s="18" t="n">
-        <f aca="false">-(D23-C23)</f>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>440</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <f aca="false">-(BILAN!D23-BILAN!C23)</f>
         <v>-23030545.0991249</v>
       </c>
-      <c r="E111" s="18" t="n">
-        <f aca="false">-(E23-D23)</f>
+      <c r="E10" s="18" t="n">
+        <f aca="false">-(BILAN!E23-BILAN!D23)</f>
         <v>-23765097.0549563</v>
       </c>
-      <c r="F111" s="18" t="n">
-        <f aca="false">-(F23-E23)</f>
+      <c r="F10" s="18" t="n">
+        <f aca="false">-(BILAN!F23-BILAN!E23)</f>
         <v>-24953351.9077041</v>
       </c>
-      <c r="G111" s="18" t="n">
-        <f aca="false">-(G23-F23)</f>
+      <c r="G10" s="18" t="n">
+        <f aca="false">-(BILAN!G23-BILAN!F23)</f>
         <v>-26201019.5030894</v>
       </c>
-      <c r="H111" s="18" t="n">
-        <f aca="false">-(H23-G23)</f>
+      <c r="H10" s="18" t="n">
+        <f aca="false">-(BILAN!H23-BILAN!G23)</f>
         <v>-27511070.4782436</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="13" t="s">
-        <v>437</v>
-      </c>
-      <c r="B112" s="12" t="s">
-        <v>438</v>
-      </c>
-      <c r="C112" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D112" s="18" t="n">
-        <f aca="false">(D55-D49)-(C55-C49)</f>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>441</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>442</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <f aca="false">(BILAN!D55-BILAN!D49)-(BILAN!C55-BILAN!C49)</f>
         <v>6230577.76672882</v>
       </c>
-      <c r="E112" s="18" t="n">
-        <f aca="false">(E55-E49)-(D55-D49)</f>
+      <c r="E11" s="18" t="n">
+        <f aca="false">(BILAN!E55-BILAN!E49)-(BILAN!D55-BILAN!D49)</f>
         <v>9162632.79350314</v>
       </c>
-      <c r="F112" s="18" t="n">
-        <f aca="false">(F55-F49)-(E55-E49)</f>
+      <c r="F11" s="18" t="n">
+        <f aca="false">(BILAN!F55-BILAN!F49)-(BILAN!E55-BILAN!E49)</f>
         <v>10558486.3890116</v>
       </c>
-      <c r="G112" s="18" t="n">
-        <f aca="false">(G55-G49)-(F55-F49)</f>
+      <c r="G11" s="18" t="n">
+        <f aca="false">(BILAN!G55-BILAN!G49)-(BILAN!F55-BILAN!F49)</f>
         <v>11329988.5599622</v>
       </c>
-      <c r="H112" s="18" t="n">
-        <f aca="false">(H55-H49)-(G55-G49)</f>
+      <c r="H11" s="18" t="n">
+        <f aca="false">(BILAN!H55-BILAN!H49)-(BILAN!G55-BILAN!G49)</f>
         <v>13990687.6879603</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="34" t="s">
-        <v>439</v>
-      </c>
-      <c r="B113" s="34" t="s">
-        <v>440</v>
-      </c>
-      <c r="C113" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D113" s="35" t="n">
-        <f aca="false">D108+D109+D110+D111+D112</f>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="34" t="s">
+        <v>443</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>444</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <f aca="false">D7+D8+D9+D10+D11</f>
         <v>156427853.275421</v>
       </c>
-      <c r="E113" s="35" t="n">
-        <f aca="false">E108+E109+E110+E111+E112</f>
+      <c r="E12" s="35" t="n">
+        <f aca="false">E7+E8+E9+E10+E11</f>
         <v>169782205.425588</v>
       </c>
-      <c r="F113" s="35" t="n">
-        <f aca="false">F108+F109+F110+F111+F112</f>
+      <c r="F12" s="35" t="n">
+        <f aca="false">F7+F8+F9+F10+F11</f>
         <v>179795401.7857</v>
       </c>
-      <c r="G113" s="35" t="n">
-        <f aca="false">G108+G109+G110+G111+G112</f>
+      <c r="G12" s="35" t="n">
+        <f aca="false">G7+G8+G9+G10+G11</f>
         <v>187705865.063985</v>
       </c>
-      <c r="H113" s="35" t="n">
-        <f aca="false">H108+H109+H110+H111+H112</f>
+      <c r="H12" s="35" t="n">
+        <f aca="false">H7+H8+H9+H10+H11</f>
         <v>195768273.654685</v>
       </c>
-      <c r="I113" s="38"/>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="13" t="s">
-        <v>441</v>
-      </c>
-      <c r="B114" s="12" t="s">
-        <v>442</v>
-      </c>
-      <c r="C114" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D114" s="15" t="n">
+      <c r="I12" s="38"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D13" s="15" t="n">
         <f aca="false">-((SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AD"))-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AD")))</f>
         <v>-0</v>
       </c>
-      <c r="E114" s="15" t="n">
+      <c r="E13" s="15" t="n">
         <f aca="false">-((SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AD"))-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AD")))</f>
         <v>-0</v>
       </c>
-      <c r="F114" s="15" t="n">
+      <c r="F13" s="15" t="n">
         <f aca="false">-((SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AD"))-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AD")))</f>
         <v>-0</v>
       </c>
-      <c r="G114" s="15" t="n">
+      <c r="G13" s="15" t="n">
         <f aca="false">-((SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AD"))-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AD")))</f>
         <v>-0</v>
       </c>
-      <c r="H114" s="15" t="n">
+      <c r="H13" s="15" t="n">
         <f aca="false">-((SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AD"))-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AD")))</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="13" t="s">
-        <v>443</v>
-      </c>
-      <c r="B115" s="12" t="s">
-        <v>444</v>
-      </c>
-      <c r="C115" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D115" s="15" t="n">
-        <f aca="false">-((SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AP")))+(D49-C49)</f>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="C14" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">-((SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$D:$D,BALANCES!$C:$C,"AP")))+(BILAN!D49-BILAN!C49)</f>
         <v>-207896547</v>
       </c>
-      <c r="E115" s="15" t="n">
-        <f aca="false">-((SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AP")))+(E49-D49)</f>
+      <c r="E14" s="15" t="n">
+        <f aca="false">-((SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$F:$F,BALANCES!$C:$C,"AP")))+(BILAN!E49-BILAN!D49)</f>
         <v>-35000000</v>
       </c>
-      <c r="F115" s="15" t="n">
-        <f aca="false">-((SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AP")))+(F49-E49)</f>
+      <c r="F14" s="15" t="n">
+        <f aca="false">-((SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$H:$H,BALANCES!$C:$C,"AP")))+(BILAN!F49-BILAN!E49)</f>
         <v>-35000000</v>
       </c>
-      <c r="G115" s="15" t="n">
-        <f aca="false">-((SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AP")))+(G49-F49)</f>
+      <c r="G14" s="15" t="n">
+        <f aca="false">-((SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$J:$J,BALANCES!$C:$C,"AP")))+(BILAN!G49-BILAN!F49)</f>
         <v>-75000000</v>
       </c>
-      <c r="H115" s="15" t="n">
-        <f aca="false">-((SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AP")))+(H49-G49)</f>
+      <c r="H14" s="15" t="n">
+        <f aca="false">-((SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$N:$N,BALANCES!$C:$C,"AP"))-(SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AJ")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AK")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AL")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AM")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AN")+SUMIFS(BALANCES!$L:$L,BALANCES!$C:$C,"AP")))+(BILAN!H49-BILAN!G49)</f>
         <v>-35000000</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="13" t="s">
-        <v>445</v>
-      </c>
-      <c r="B116" s="12" t="s">
-        <v>446</v>
-      </c>
-      <c r="C116" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D116" s="18" t="n">
-        <f aca="false">-(D16-C16)</f>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>449</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>450</v>
+      </c>
+      <c r="C15" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <f aca="false">-(BILAN!D16-BILAN!C16)</f>
         <v>-0</v>
       </c>
-      <c r="E116" s="18" t="n">
-        <f aca="false">-(E16-D16)</f>
+      <c r="E15" s="18" t="n">
+        <f aca="false">-(BILAN!E16-BILAN!D16)</f>
         <v>-0</v>
       </c>
-      <c r="F116" s="18" t="n">
-        <f aca="false">-(F16-E16)</f>
+      <c r="F15" s="18" t="n">
+        <f aca="false">-(BILAN!F16-BILAN!E16)</f>
         <v>-0</v>
       </c>
-      <c r="G116" s="18" t="n">
-        <f aca="false">-(G16-F16)</f>
+      <c r="G15" s="18" t="n">
+        <f aca="false">-(BILAN!G16-BILAN!F16)</f>
         <v>-0</v>
       </c>
-      <c r="H116" s="18" t="n">
-        <f aca="false">-(H16-G16)</f>
+      <c r="H15" s="18" t="n">
+        <f aca="false">-(BILAN!H16-BILAN!G16)</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="13" t="s">
-        <v>447</v>
-      </c>
-      <c r="B117" s="12" t="s">
-        <v>448</v>
-      </c>
-      <c r="C117" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D117" s="18" t="n">
-        <f aca="false">D97</f>
-        <v>0</v>
-      </c>
-      <c r="E117" s="18" t="n">
-        <f aca="false">E97</f>
-        <v>0</v>
-      </c>
-      <c r="F117" s="18" t="n">
-        <f aca="false">F97</f>
-        <v>0</v>
-      </c>
-      <c r="G117" s="18" t="n">
-        <f aca="false">G97</f>
-        <v>0</v>
-      </c>
-      <c r="H117" s="18" t="n">
-        <f aca="false">H97</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="13" t="s">
-        <v>449</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>450</v>
-      </c>
-      <c r="C118" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D118" s="18" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>451</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>452</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!D40</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!E40</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!F40</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!G40</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!H40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>454</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D17" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E118" s="18" t="n">
+      <c r="E17" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F118" s="18" t="n">
+      <c r="F17" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G118" s="18" t="n">
+      <c r="G17" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="H118" s="18" t="n">
+      <c r="H17" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="34" t="s">
-        <v>451</v>
-      </c>
-      <c r="B119" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="C119" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D119" s="35" t="n">
-        <f aca="false">D114+D115+D116+D117+D118</f>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="34" t="s">
+        <v>455</v>
+      </c>
+      <c r="B18" s="34" t="s">
+        <v>456</v>
+      </c>
+      <c r="C18" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <f aca="false">D13+D14+D15+D16+D17</f>
         <v>-207896547</v>
       </c>
-      <c r="E119" s="35" t="n">
-        <f aca="false">E114+E115+E116+E117+E118</f>
+      <c r="E18" s="35" t="n">
+        <f aca="false">E13+E14+E15+E16+E17</f>
         <v>-35000000</v>
       </c>
-      <c r="F119" s="35" t="n">
-        <f aca="false">F114+F115+F116+F117+F118</f>
+      <c r="F18" s="35" t="n">
+        <f aca="false">F13+F14+F15+F16+F17</f>
         <v>-35000000</v>
       </c>
-      <c r="G119" s="35" t="n">
-        <f aca="false">G114+G115+G116+G117+G118</f>
+      <c r="G18" s="35" t="n">
+        <f aca="false">G13+G14+G15+G16+G17</f>
         <v>-75000000</v>
       </c>
-      <c r="H119" s="35" t="n">
-        <f aca="false">H114+H115+H116+H117+H118</f>
+      <c r="H18" s="35" t="n">
+        <f aca="false">H13+H14+H15+H16+H17</f>
         <v>-35000000</v>
       </c>
-      <c r="I119" s="38"/>
-    </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="13" t="s">
-        <v>453</v>
-      </c>
-      <c r="B120" s="12" t="s">
-        <v>454</v>
-      </c>
-      <c r="C120" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D120" s="18" t="n">
-        <f aca="false">D33-C33</f>
-        <v>0</v>
-      </c>
-      <c r="E120" s="18" t="n">
-        <f aca="false">E33-D33</f>
-        <v>0</v>
-      </c>
-      <c r="F120" s="18" t="n">
-        <f aca="false">F33-E33</f>
-        <v>0</v>
-      </c>
-      <c r="G120" s="18" t="n">
-        <f aca="false">G33-F33</f>
-        <v>0</v>
-      </c>
-      <c r="H120" s="18" t="n">
-        <f aca="false">H33-G33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="13" t="s">
-        <v>455</v>
-      </c>
-      <c r="B121" s="12" t="s">
-        <v>456</v>
-      </c>
-      <c r="C121" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D121" s="18" t="n">
-        <f aca="false">D41-C41</f>
-        <v>0</v>
-      </c>
-      <c r="E121" s="18" t="n">
-        <f aca="false">E41-D41</f>
-        <v>0</v>
-      </c>
-      <c r="F121" s="18" t="n">
-        <f aca="false">F41-E41</f>
-        <v>0</v>
-      </c>
-      <c r="G121" s="18" t="n">
-        <f aca="false">G41-F41</f>
-        <v>0</v>
-      </c>
-      <c r="H121" s="18" t="n">
-        <f aca="false">H41-G41</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="13" t="s">
+      <c r="I18" s="38"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
         <v>457</v>
       </c>
-      <c r="B122" s="12" t="s">
+      <c r="B19" s="12" t="s">
         <v>458</v>
       </c>
-      <c r="C122" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D122" s="18" t="n">
+      <c r="C19" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <f aca="false">BILAN!D33-BILAN!C33</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <f aca="false">BILAN!E33-BILAN!D33</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <f aca="false">BILAN!F33-BILAN!E33</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <f aca="false">BILAN!G33-BILAN!F33</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="18" t="n">
+        <f aca="false">BILAN!H33-BILAN!G33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>460</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">BILAN!D41-BILAN!C41</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <f aca="false">BILAN!E41-BILAN!D41</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <f aca="false">BILAN!F41-BILAN!E41</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <f aca="false">BILAN!G41-BILAN!F41</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="18" t="n">
+        <f aca="false">BILAN!H41-BILAN!G41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>462</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D21" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E122" s="18" t="n">
+      <c r="E21" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F122" s="18" t="n">
+      <c r="F21" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G122" s="18" t="n">
+      <c r="G21" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="H122" s="18" t="n">
+      <c r="H21" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="13" t="s">
-        <v>459</v>
-      </c>
-      <c r="B123" s="12" t="s">
-        <v>460</v>
-      </c>
-      <c r="C123" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D123" s="18" t="n">
-        <f aca="false">-((C37+C38+C39+C40)-(D37+D38+D39))</f>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>463</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>464</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <f aca="false">-((BILAN!C37+BILAN!C38+BILAN!C39+BILAN!C40)-(BILAN!D37+BILAN!D38+BILAN!D39))</f>
         <v>-0</v>
       </c>
-      <c r="E123" s="18" t="n">
-        <f aca="false">-((D37+D38+D39+D40)-(E37+E38+E39))</f>
+      <c r="E22" s="18" t="n">
+        <f aca="false">-((BILAN!D37+BILAN!D38+BILAN!D39+BILAN!D40)-(BILAN!E37+BILAN!E38+BILAN!E39))</f>
         <v>-0</v>
       </c>
-      <c r="F123" s="18" t="n">
-        <f aca="false">-((E37+E38+E39+E40)-(F37+F38+F39))</f>
+      <c r="F22" s="18" t="n">
+        <f aca="false">-((BILAN!E37+BILAN!E38+BILAN!E39+BILAN!E40)-(BILAN!F37+BILAN!F38+BILAN!F39))</f>
         <v>-0</v>
       </c>
-      <c r="G123" s="18" t="n">
-        <f aca="false">-((F37+F38+F39+F40)-(G37+G38+G39))</f>
+      <c r="G22" s="18" t="n">
+        <f aca="false">-((BILAN!F37+BILAN!F38+BILAN!F39+BILAN!F40)-(BILAN!G37+BILAN!G38+BILAN!G39))</f>
         <v>-0</v>
       </c>
-      <c r="H123" s="18" t="n">
-        <f aca="false">-((G37+G38+G39+G40)-(H37+H38+H39))</f>
+      <c r="H22" s="18" t="n">
+        <f aca="false">-((BILAN!G37+BILAN!G38+BILAN!G39+BILAN!G40)-(BILAN!H37+BILAN!H38+BILAN!H39))</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="34" t="s">
-        <v>461</v>
-      </c>
-      <c r="B124" s="34" t="s">
-        <v>462</v>
-      </c>
-      <c r="C124" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D124" s="35" t="n">
-        <f aca="false">D120+D121+D122+D123</f>
-        <v>0</v>
-      </c>
-      <c r="E124" s="35" t="n">
-        <f aca="false">E120+E121+E122+E123</f>
-        <v>0</v>
-      </c>
-      <c r="F124" s="35" t="n">
-        <f aca="false">F120+F121+F122+F123</f>
-        <v>0</v>
-      </c>
-      <c r="G124" s="35" t="n">
-        <f aca="false">G120+G121+G122+G123</f>
-        <v>0</v>
-      </c>
-      <c r="H124" s="35" t="n">
-        <f aca="false">H120+H121+H122+H123</f>
-        <v>0</v>
-      </c>
-      <c r="I124" s="38"/>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="13" t="s">
-        <v>463</v>
-      </c>
-      <c r="B125" s="12" t="s">
-        <v>464</v>
-      </c>
-      <c r="C125" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D125" s="15" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="34" t="s">
+        <v>465</v>
+      </c>
+      <c r="B23" s="34" t="s">
+        <v>466</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D23" s="35" t="n">
+        <f aca="false">D19+D20+D21+D22</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="35" t="n">
+        <f aca="false">E19+E20+E21+E22</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="35" t="n">
+        <f aca="false">F19+F20+F21+F22</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="35" t="n">
+        <f aca="false">G19+G20+G21+G22</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="35" t="n">
+        <f aca="false">H19+H20+H21+H22</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="38"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D24" s="15" t="n">
         <f aca="false">HYPOTHESES!D41</f>
         <v>0</v>
       </c>
-      <c r="E125" s="15" t="n">
+      <c r="E24" s="15" t="n">
         <f aca="false">HYPOTHESES!E41</f>
         <v>0</v>
       </c>
-      <c r="F125" s="15" t="n">
+      <c r="F24" s="15" t="n">
         <f aca="false">HYPOTHESES!F41</f>
         <v>0</v>
       </c>
-      <c r="G125" s="15" t="n">
+      <c r="G24" s="15" t="n">
         <f aca="false">HYPOTHESES!G41</f>
         <v>0</v>
       </c>
-      <c r="H125" s="15" t="n">
+      <c r="H24" s="15" t="n">
         <f aca="false">HYPOTHESES!H41</f>
         <v>0</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="13" t="s">
-        <v>465</v>
-      </c>
-      <c r="B126" s="12" t="s">
-        <v>466</v>
-      </c>
-      <c r="C126" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D126" s="18" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>470</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D25" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E126" s="18" t="n">
+      <c r="E25" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F126" s="18" t="n">
+      <c r="F25" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G126" s="18" t="n">
+      <c r="G25" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="H126" s="18" t="n">
+      <c r="H25" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="13" t="s">
-        <v>467</v>
-      </c>
-      <c r="B127" s="12" t="s">
-        <v>468</v>
-      </c>
-      <c r="C127" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D127" s="15" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>471</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>472</v>
+      </c>
+      <c r="C26" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D26" s="15" t="n">
         <f aca="false">-(HYPOTHESES!D42+HYPOTHESES!D43)</f>
         <v>-30449110</v>
       </c>
-      <c r="E127" s="15" t="n">
+      <c r="E26" s="15" t="n">
         <f aca="false">-(HYPOTHESES!E42+HYPOTHESES!E43)</f>
         <v>-19829416</v>
       </c>
-      <c r="F127" s="15" t="n">
+      <c r="F26" s="15" t="n">
         <f aca="false">-(HYPOTHESES!F42+HYPOTHESES!F43)</f>
         <v>-0</v>
       </c>
-      <c r="G127" s="15" t="n">
+      <c r="G26" s="15" t="n">
         <f aca="false">-(HYPOTHESES!G42+HYPOTHESES!G43)</f>
         <v>-0</v>
       </c>
-      <c r="H127" s="15" t="n">
+      <c r="H26" s="15" t="n">
         <f aca="false">-(HYPOTHESES!H42+HYPOTHESES!H43)</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="34" t="s">
-        <v>469</v>
-      </c>
-      <c r="B128" s="34" t="s">
-        <v>470</v>
-      </c>
-      <c r="C128" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D128" s="35" t="n">
-        <f aca="false">D125+D126+D127</f>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="34" t="s">
+        <v>473</v>
+      </c>
+      <c r="B27" s="34" t="s">
+        <v>474</v>
+      </c>
+      <c r="C27" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D27" s="35" t="n">
+        <f aca="false">D24+D25+D26</f>
         <v>-30449110</v>
       </c>
-      <c r="E128" s="35" t="n">
-        <f aca="false">E125+E126+E127</f>
+      <c r="E27" s="35" t="n">
+        <f aca="false">E24+E25+E26</f>
         <v>-19829416</v>
       </c>
-      <c r="F128" s="35" t="n">
-        <f aca="false">F125+F126+F127</f>
-        <v>0</v>
-      </c>
-      <c r="G128" s="35" t="n">
-        <f aca="false">G125+G126+G127</f>
-        <v>0</v>
-      </c>
-      <c r="H128" s="35" t="n">
-        <f aca="false">H125+H126+H127</f>
-        <v>0</v>
-      </c>
-      <c r="I128" s="38"/>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="34" t="s">
-        <v>471</v>
-      </c>
-      <c r="B129" s="34" t="s">
-        <v>472</v>
-      </c>
-      <c r="C129" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D129" s="35" t="n">
-        <f aca="false">D124+D128</f>
+      <c r="F27" s="35" t="n">
+        <f aca="false">F24+F25+F26</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="35" t="n">
+        <f aca="false">G24+G25+G26</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="35" t="n">
+        <f aca="false">H24+H25+H26</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="34" t="s">
+        <v>475</v>
+      </c>
+      <c r="B28" s="34" t="s">
+        <v>476</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D28" s="35" t="n">
+        <f aca="false">D23+D27</f>
         <v>-30449110</v>
       </c>
-      <c r="E129" s="35" t="n">
-        <f aca="false">E124+E128</f>
+      <c r="E28" s="35" t="n">
+        <f aca="false">E23+E27</f>
         <v>-19829416</v>
       </c>
-      <c r="F129" s="35" t="n">
-        <f aca="false">F124+F128</f>
-        <v>0</v>
-      </c>
-      <c r="G129" s="35" t="n">
-        <f aca="false">G124+G128</f>
-        <v>0</v>
-      </c>
-      <c r="H129" s="35" t="n">
-        <f aca="false">H124+H128</f>
-        <v>0</v>
-      </c>
-      <c r="I129" s="38"/>
-    </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="34" t="s">
-        <v>473</v>
-      </c>
-      <c r="B130" s="34" t="s">
-        <v>474</v>
-      </c>
-      <c r="C130" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D130" s="35" t="n">
-        <f aca="false">D113+D119+D129</f>
+      <c r="F28" s="35" t="n">
+        <f aca="false">F23+F27</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="35" t="n">
+        <f aca="false">G23+G27</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="35" t="n">
+        <f aca="false">H23+H27</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="38"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="34" t="s">
+        <v>477</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D29" s="35" t="n">
+        <f aca="false">D12+D18+D28</f>
         <v>-81917803.7245795</v>
       </c>
-      <c r="E130" s="35" t="n">
-        <f aca="false">E113+E119+E129</f>
+      <c r="E29" s="35" t="n">
+        <f aca="false">E12+E18+E28</f>
         <v>114952789.425588</v>
       </c>
-      <c r="F130" s="35" t="n">
-        <f aca="false">F113+F119+F129</f>
+      <c r="F29" s="35" t="n">
+        <f aca="false">F12+F18+F28</f>
         <v>144795401.7857</v>
       </c>
-      <c r="G130" s="35" t="n">
-        <f aca="false">G113+G119+G129</f>
+      <c r="G29" s="35" t="n">
+        <f aca="false">G12+G18+G28</f>
         <v>112705865.063985</v>
       </c>
-      <c r="H130" s="35" t="n">
-        <f aca="false">H113+H119+H129</f>
+      <c r="H29" s="35" t="n">
+        <f aca="false">H12+H18+H28</f>
         <v>160768273.654685</v>
       </c>
-      <c r="I130" s="38"/>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="34" t="s">
-        <v>475</v>
-      </c>
-      <c r="B131" s="34" t="s">
-        <v>476</v>
-      </c>
-      <c r="C131" s="40" t="s">
-        <v>428</v>
-      </c>
-      <c r="D131" s="35" t="n">
-        <f aca="false">D130+D107</f>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="B30" s="34" t="s">
+        <v>480</v>
+      </c>
+      <c r="C30" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="D30" s="35" t="n">
+        <f aca="false">D29+D6</f>
         <v>46216154.2754206</v>
       </c>
-      <c r="E131" s="35" t="n">
-        <f aca="false">E130+E107</f>
+      <c r="E30" s="35" t="n">
+        <f aca="false">E29+E6</f>
         <v>161168943.701008</v>
       </c>
-      <c r="F131" s="35" t="n">
-        <f aca="false">F130+F107</f>
+      <c r="F30" s="35" t="n">
+        <f aca="false">F29+F6</f>
         <v>305964345.486709</v>
       </c>
-      <c r="G131" s="35" t="n">
-        <f aca="false">G130+G107</f>
+      <c r="G30" s="35" t="n">
+        <f aca="false">G29+G6</f>
         <v>418670210.550694</v>
       </c>
-      <c r="H131" s="35" t="n">
-        <f aca="false">H130+H107</f>
+      <c r="H30" s="35" t="n">
+        <f aca="false">H29+H6</f>
         <v>579438484.205379</v>
       </c>
-      <c r="I131" s="38"/>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B132" s="7" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="36" t="s">
+      <c r="I30" s="38"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="7" t="s">
+        <v>481</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFC00000"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="str">
+        <f aca="false">"Entité : "&amp;HYPOTHESES!$C$4</f>
+        <v>Entité : MON ENTREPRISE</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="36" t="s">
         <v>265</v>
       </c>
-      <c r="B134" s="36" t="s">
-        <v>478</v>
-      </c>
-      <c r="C134" s="36" t="str">
+      <c r="B5" s="36" t="s">
+        <v>484</v>
+      </c>
+      <c r="C5" s="36" t="str">
         <f aca="false">"Réel "&amp;HYPOTHESES!$C$5</f>
         <v>Réel 2024</v>
       </c>
-      <c r="D134" s="37" t="n">
+      <c r="D5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+1</f>
         <v>2025</v>
       </c>
-      <c r="E134" s="37" t="n">
+      <c r="E5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+2</f>
         <v>2026</v>
       </c>
-      <c r="F134" s="37" t="n">
+      <c r="F5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+3</f>
         <v>2027</v>
       </c>
-      <c r="G134" s="37" t="n">
+      <c r="G5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+4</f>
         <v>2028</v>
       </c>
-      <c r="H134" s="37" t="n">
+      <c r="H5" s="37" t="n">
         <f aca="false">HYPOTHESES!$C$5+5</f>
         <v>2029</v>
       </c>
-      <c r="I134" s="36" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="13"/>
-      <c r="B135" s="12" t="s">
-        <v>479</v>
-      </c>
-      <c r="C135" s="42" t="str">
+      <c r="I5" s="36" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13"/>
+      <c r="B6" s="12" t="s">
+        <v>486</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <f aca="false">BALANCES!D92</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">BALANCES!F92</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">BALANCES!H92</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <f aca="false">BALANCES!J92</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">BALANCES!L92</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <f aca="false">BALANCES!N92</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13"/>
+      <c r="B7" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <f aca="false">BILAN!C30-BILAN!C60</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <f aca="false">BILAN!D30-BILAN!D60</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <f aca="false">BILAN!E30-BILAN!E60</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <f aca="false">BILAN!F30-BILAN!F60</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <f aca="false">BILAN!G30-BILAN!G60</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="18" t="n">
+        <f aca="false">BILAN!H30-BILAN!H60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13"/>
+      <c r="B8" s="12" t="s">
+        <v>488</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!C47-HYPOTHESES!C92</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!D47-HYPOTHESES!D92</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!E47-HYPOTHESES!E92</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!F47-HYPOTHESES!F92</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!G47-HYPOTHESES!G92</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <f aca="false">'COMPTE DE RESULTAT'!H47-HYPOTHESES!H92</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13"/>
+      <c r="B9" s="12" t="s">
+        <v>489</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <f aca="false">TFT!D30-(BILAN!D28-BILAN!D58)</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <f aca="false">TFT!E30-(BILAN!E28-BILAN!E58)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <f aca="false">TFT!F30-(BILAN!F28-BILAN!F58)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <f aca="false">TFT!G30-(BILAN!G28-BILAN!G58)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <f aca="false">TFT!H30-(BILAN!H28-BILAN!H58)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+      <c r="B10" s="12" t="s">
+        <v>490</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <f aca="false">BILAN!D43-(BILAN!C43+'COMPTE DE RESULTAT'!D47+TFT!D22+TFT!D19+TFT!D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <f aca="false">BILAN!E43-(BILAN!D43+'COMPTE DE RESULTAT'!E47+TFT!E22+TFT!E19+TFT!E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <f aca="false">BILAN!F43-(BILAN!E43+'COMPTE DE RESULTAT'!F47+TFT!F22+TFT!F19+TFT!F20)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <f aca="false">BILAN!G43-(BILAN!F43+'COMPTE DE RESULTAT'!G47+TFT!G22+TFT!G19+TFT!G20)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <f aca="false">BILAN!H43-(BILAN!G43+'COMPTE DE RESULTAT'!H47+TFT!H22+TFT!H19+TFT!H20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13"/>
+      <c r="B11" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>432</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <f aca="false">TFT!D6-(BILAN!C28-BILAN!C58)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <f aca="false">TFT!E6-(BILAN!D28-BILAN!D58)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <f aca="false">TFT!F6-(BILAN!E28-BILAN!E58)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <f aca="false">TFT!G6-(BILAN!F28-BILAN!F58)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="18" t="n">
+        <f aca="false">TFT!H6-(BILAN!G28-BILAN!G58)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13"/>
+      <c r="B12" s="12" t="s">
+        <v>492</v>
+      </c>
+      <c r="C12" s="32" t="n">
+        <f aca="false">IF(BILAN!C28-BILAN!C58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <f aca="false">IF(BILAN!D28-BILAN!D58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <f aca="false">IF(BILAN!E28-BILAN!E58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <f aca="false">IF(BILAN!F28-BILAN!F58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <f aca="false">IF(BILAN!G28-BILAN!G58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <f aca="false">IF(BILAN!H28-BILAN!H58&lt;0,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13"/>
+      <c r="B13" s="12" t="s">
+        <v>493</v>
+      </c>
+      <c r="C13" s="32" t="n">
+        <f aca="false">IF(BILAN!C43&lt;BILAN!C33/2,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <f aca="false">IF(BILAN!D43&lt;BILAN!D33/2,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="32" t="n">
+        <f aca="false">IF(BILAN!E43&lt;BILAN!E33/2,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="32" t="n">
+        <f aca="false">IF(BILAN!F43&lt;BILAN!F33/2,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="32" t="n">
+        <f aca="false">IF(BILAN!G43&lt;BILAN!G33/2,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="32" t="n">
+        <f aca="false">IF(BILAN!H43&lt;BILAN!H33/2,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="42" t="s">
+        <v>494</v>
+      </c>
+      <c r="C14" s="43" t="n">
+        <f aca="false">COUNTIF(C6:C13,"&gt;0.5")+COUNTIF(C6:C13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="43" t="n">
+        <f aca="false">COUNTIF(D6:D13,"&gt;0.5")+COUNTIF(D6:D13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="43" t="n">
+        <f aca="false">COUNTIF(E6:E13,"&gt;0.5")+COUNTIF(E6:E13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="43" t="n">
+        <f aca="false">COUNTIF(F6:F13,"&gt;0.5")+COUNTIF(F6:F13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="43" t="n">
+        <f aca="false">COUNTIF(G6:G13,"&gt;0.5")+COUNTIF(G6:G13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="43" t="n">
+        <f aca="false">COUNTIF(H6:H13,"&gt;0.5")+COUNTIF(H6:H13,"&lt;-0.5")</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="42" t="str">
+        <f aca="false">IF(SUM(C14:H14)=0,"OK","À VÉRIFIER")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>495</v>
+      </c>
+      <c r="C16" s="36" t="str">
+        <f aca="false">"Réel "&amp;HYPOTHESES!$C$5</f>
+        <v>Réel 2024</v>
+      </c>
+      <c r="D16" s="37" t="n">
+        <f aca="false">HYPOTHESES!$C$5+1</f>
+        <v>2025</v>
+      </c>
+      <c r="E16" s="37" t="n">
+        <f aca="false">HYPOTHESES!$C$5+2</f>
+        <v>2026</v>
+      </c>
+      <c r="F16" s="37" t="n">
+        <f aca="false">HYPOTHESES!$C$5+3</f>
+        <v>2027</v>
+      </c>
+      <c r="G16" s="37" t="n">
+        <f aca="false">HYPOTHESES!$C$5+4</f>
+        <v>2028</v>
+      </c>
+      <c r="H16" s="37" t="n">
+        <f aca="false">HYPOTHESES!$C$5+5</f>
+        <v>2029</v>
+      </c>
+      <c r="I16" s="36" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+      <c r="B17" s="12" t="s">
+        <v>496</v>
+      </c>
+      <c r="C17" s="44" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="D135" s="42" t="n">
-        <f aca="false">IF(C70=0,0,D70/C70-1)</f>
+      <c r="D17" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!C13=0,0,'COMPTE DE RESULTAT'!D13/'COMPTE DE RESULTAT'!C13-1)</f>
         <v>0.05</v>
       </c>
-      <c r="E135" s="42" t="n">
-        <f aca="false">IF(D70=0,0,E70/D70-1)</f>
+      <c r="E17" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!D13=0,0,'COMPTE DE RESULTAT'!E13/'COMPTE DE RESULTAT'!D13-1)</f>
         <v>0.05</v>
       </c>
-      <c r="F135" s="42" t="n">
-        <f aca="false">IF(E70=0,0,F70/E70-1)</f>
+      <c r="F17" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!E13=0,0,'COMPTE DE RESULTAT'!F13/'COMPTE DE RESULTAT'!E13-1)</f>
         <v>0.05</v>
       </c>
-      <c r="G135" s="42" t="n">
-        <f aca="false">IF(F70=0,0,G70/F70-1)</f>
+      <c r="G17" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!F13=0,0,'COMPTE DE RESULTAT'!G13/'COMPTE DE RESULTAT'!F13-1)</f>
         <v>0.05</v>
       </c>
-      <c r="H135" s="42" t="n">
-        <f aca="false">IF(G70=0,0,H70/G70-1)</f>
+      <c r="H17" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!G13=0,0,'COMPTE DE RESULTAT'!H13/'COMPTE DE RESULTAT'!G13-1)</f>
         <v>0.05</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="13"/>
-      <c r="B136" s="12" t="s">
-        <v>480</v>
-      </c>
-      <c r="C136" s="42" t="n">
-        <f aca="false">IF(C70=0,0,C84/C70)</f>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13"/>
+      <c r="B18" s="12" t="s">
+        <v>497</v>
+      </c>
+      <c r="C18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!C13=0,0,'COMPTE DE RESULTAT'!C27/'COMPTE DE RESULTAT'!C13)</f>
         <v>0.422394255613904</v>
       </c>
-      <c r="D136" s="42" t="n">
-        <f aca="false">IF(D70=0,0,D84/D70)</f>
+      <c r="D18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!D13=0,0,'COMPTE DE RESULTAT'!D27/'COMPTE DE RESULTAT'!D13)</f>
         <v>0.4224</v>
       </c>
-      <c r="E136" s="42" t="n">
-        <f aca="false">IF(E70=0,0,E84/E70)</f>
+      <c r="E18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!E13=0,0,'COMPTE DE RESULTAT'!E27/'COMPTE DE RESULTAT'!E13)</f>
         <v>0.4224</v>
       </c>
-      <c r="F136" s="42" t="n">
-        <f aca="false">IF(F70=0,0,F84/F70)</f>
+      <c r="F18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!F13=0,0,'COMPTE DE RESULTAT'!F27/'COMPTE DE RESULTAT'!F13)</f>
         <v>0.4224</v>
       </c>
-      <c r="G136" s="42" t="n">
-        <f aca="false">IF(G70=0,0,G84/G70)</f>
+      <c r="G18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!G13=0,0,'COMPTE DE RESULTAT'!G27/'COMPTE DE RESULTAT'!G13)</f>
         <v>0.4224</v>
       </c>
-      <c r="H136" s="42" t="n">
-        <f aca="false">IF(H70=0,0,H84/H70)</f>
+      <c r="H18" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!H13=0,0,'COMPTE DE RESULTAT'!H27/'COMPTE DE RESULTAT'!H13)</f>
         <v>0.4224</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="13"/>
-      <c r="B137" s="12" t="s">
-        <v>481</v>
-      </c>
-      <c r="C137" s="42" t="n">
-        <f aca="false">IF(C70=0,0,C86/C70)</f>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+      <c r="B19" s="12" t="s">
+        <v>498</v>
+      </c>
+      <c r="C19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!C13=0,0,'COMPTE DE RESULTAT'!C29/'COMPTE DE RESULTAT'!C13)</f>
         <v>0.271151063655286</v>
       </c>
-      <c r="D137" s="42" t="n">
-        <f aca="false">IF(D70=0,0,D86/D70)</f>
+      <c r="D19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!D13=0,0,'COMPTE DE RESULTAT'!D29/'COMPTE DE RESULTAT'!D13)</f>
         <v>0.2712</v>
       </c>
-      <c r="E137" s="42" t="n">
-        <f aca="false">IF(E70=0,0,E86/E70)</f>
+      <c r="E19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!E13=0,0,'COMPTE DE RESULTAT'!E29/'COMPTE DE RESULTAT'!E13)</f>
         <v>0.2712</v>
       </c>
-      <c r="F137" s="42" t="n">
-        <f aca="false">IF(F70=0,0,F86/F70)</f>
+      <c r="F19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!F13=0,0,'COMPTE DE RESULTAT'!F29/'COMPTE DE RESULTAT'!F13)</f>
         <v>0.2712</v>
       </c>
-      <c r="G137" s="42" t="n">
-        <f aca="false">IF(G70=0,0,G86/G70)</f>
+      <c r="G19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!G13=0,0,'COMPTE DE RESULTAT'!G29/'COMPTE DE RESULTAT'!G13)</f>
         <v>0.2712</v>
       </c>
-      <c r="H137" s="42" t="n">
-        <f aca="false">IF(H70=0,0,H86/H70)</f>
+      <c r="H19" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!H13=0,0,'COMPTE DE RESULTAT'!H29/'COMPTE DE RESULTAT'!H13)</f>
         <v>0.2712</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="13"/>
-      <c r="B138" s="12" t="s">
-        <v>482</v>
-      </c>
-      <c r="C138" s="42" t="n">
-        <f aca="false">IF(C70=0,0,C104/C70)</f>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="B20" s="12" t="s">
+        <v>499</v>
+      </c>
+      <c r="C20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!C13=0,0,'COMPTE DE RESULTAT'!C47/'COMPTE DE RESULTAT'!C13)</f>
         <v>0.103703436001107</v>
       </c>
-      <c r="D138" s="42" t="n">
-        <f aca="false">IF(D70=0,0,D104/D70)</f>
+      <c r="D20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!D13=0,0,'COMPTE DE RESULTAT'!D47/'COMPTE DE RESULTAT'!D13)</f>
         <v>0.0946483336349708</v>
       </c>
-      <c r="E138" s="42" t="n">
-        <f aca="false">IF(E70=0,0,E104/E70)</f>
+      <c r="E20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!E13=0,0,'COMPTE DE RESULTAT'!E47/'COMPTE DE RESULTAT'!E13)</f>
         <v>0.0950332119112992</v>
       </c>
-      <c r="F138" s="42" t="n">
-        <f aca="false">IF(F70=0,0,F104/F70)</f>
+      <c r="F20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!F13=0,0,'COMPTE DE RESULTAT'!F47/'COMPTE DE RESULTAT'!F13)</f>
         <v>0.0988662760724514</v>
       </c>
-      <c r="G138" s="42" t="n">
-        <f aca="false">IF(G70=0,0,G104/G70)</f>
+      <c r="G20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!G13=0,0,'COMPTE DE RESULTAT'!G47/'COMPTE DE RESULTAT'!G13)</f>
         <v>0.103374378862353</v>
       </c>
-      <c r="H138" s="42" t="n">
-        <f aca="false">IF(H70=0,0,H104/H70)</f>
+      <c r="H20" s="44" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!H13=0,0,'COMPTE DE RESULTAT'!H47/'COMPTE DE RESULTAT'!H13)</f>
         <v>0.114689769202218</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="13"/>
-      <c r="B139" s="12" t="s">
-        <v>483</v>
-      </c>
-      <c r="C139" s="18" t="n">
-        <f aca="false">C48-C17</f>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+      <c r="B21" s="12" t="s">
+        <v>500</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <f aca="false">BILAN!C48-BILAN!C17</f>
         <v>268769832</v>
       </c>
-      <c r="D139" s="18" t="n">
-        <f aca="false">D48-D17</f>
+      <c r="D21" s="18" t="n">
+        <f aca="false">BILAN!D48-BILAN!D17</f>
         <v>336548542.607817</v>
       </c>
-      <c r="E139" s="18" t="n">
-        <f aca="false">E48-E17</f>
+      <c r="E21" s="18" t="n">
+        <f aca="false">BILAN!E48-BILAN!E17</f>
         <v>466103796.294858</v>
       </c>
-      <c r="F139" s="18" t="n">
-        <f aca="false">F48-F17</f>
+      <c r="F21" s="18" t="n">
+        <f aca="false">BILAN!F48-BILAN!F17</f>
         <v>625294063.59925</v>
       </c>
-      <c r="G139" s="18" t="n">
-        <f aca="false">G48-G17</f>
+      <c r="G21" s="18" t="n">
+        <f aca="false">BILAN!G48-BILAN!G17</f>
         <v>752870959.606363</v>
       </c>
-      <c r="H139" s="18" t="n">
-        <f aca="false">H48-H17</f>
+      <c r="H21" s="18" t="n">
+        <f aca="false">BILAN!H48-BILAN!H17</f>
         <v>927159616.051331</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="13"/>
-      <c r="B140" s="12" t="s">
-        <v>484</v>
-      </c>
-      <c r="C140" s="18" t="n">
-        <f aca="false">C24-C55</f>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+      <c r="B22" s="12" t="s">
+        <v>501</v>
+      </c>
+      <c r="C22" s="18" t="n">
+        <f aca="false">BILAN!C24-BILAN!C55</f>
         <v>140635874</v>
       </c>
-      <c r="D140" s="18" t="n">
-        <f aca="false">D24-D55</f>
+      <c r="D22" s="18" t="n">
+        <f aca="false">BILAN!D24-BILAN!D55</f>
         <v>290332388.332396</v>
       </c>
-      <c r="E140" s="18" t="n">
-        <f aca="false">E24-E55</f>
+      <c r="E22" s="18" t="n">
+        <f aca="false">BILAN!E24-BILAN!E55</f>
         <v>304934852.593849</v>
       </c>
-      <c r="F140" s="18" t="n">
-        <f aca="false">F24-F55</f>
+      <c r="F22" s="18" t="n">
+        <f aca="false">BILAN!F24-BILAN!F55</f>
         <v>319329718.112542</v>
       </c>
-      <c r="G140" s="18" t="n">
-        <f aca="false">G24-G55</f>
+      <c r="G22" s="18" t="n">
+        <f aca="false">BILAN!G24-BILAN!G55</f>
         <v>334200749.055669</v>
       </c>
-      <c r="H140" s="18" t="n">
-        <f aca="false">H24-H55</f>
+      <c r="H22" s="18" t="n">
+        <f aca="false">BILAN!H24-BILAN!H55</f>
         <v>347721131.845952</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="34"/>
-      <c r="B141" s="34" t="s">
-        <v>485</v>
-      </c>
-      <c r="C141" s="35" t="n">
-        <f aca="false">C28-C58</f>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="34"/>
+      <c r="B23" s="34" t="s">
+        <v>502</v>
+      </c>
+      <c r="C23" s="35" t="n">
+        <f aca="false">BILAN!C28-BILAN!C58</f>
         <v>128133958</v>
       </c>
-      <c r="D141" s="35" t="n">
-        <f aca="false">D28-D58</f>
+      <c r="D23" s="35" t="n">
+        <f aca="false">BILAN!D28-BILAN!D58</f>
         <v>46216154.2754206</v>
       </c>
-      <c r="E141" s="35" t="n">
-        <f aca="false">E28-E58</f>
+      <c r="E23" s="35" t="n">
+        <f aca="false">BILAN!E28-BILAN!E58</f>
         <v>161168943.701008</v>
       </c>
-      <c r="F141" s="35" t="n">
-        <f aca="false">F28-F58</f>
+      <c r="F23" s="35" t="n">
+        <f aca="false">BILAN!F28-BILAN!F58</f>
         <v>305964345.486709</v>
       </c>
-      <c r="G141" s="35" t="n">
-        <f aca="false">G28-G58</f>
+      <c r="G23" s="35" t="n">
+        <f aca="false">BILAN!G28-BILAN!G58</f>
         <v>418670210.550694</v>
       </c>
-      <c r="H141" s="35" t="n">
-        <f aca="false">H28-H58</f>
+      <c r="H23" s="35" t="n">
+        <f aca="false">BILAN!H28-BILAN!H58</f>
         <v>579438484.205379</v>
       </c>
-      <c r="I141" s="38"/>
-    </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="13"/>
-      <c r="B142" s="12" t="s">
-        <v>486</v>
-      </c>
-      <c r="C142" s="43" t="n">
-        <f aca="false">IF(C70=0,0,C140/C70*360)</f>
+      <c r="I23" s="38"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13"/>
+      <c r="B24" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="C24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!C13=0,0,C22/'COMPTE DE RESULTAT'!C13*360)</f>
         <v>72.2210937202613</v>
       </c>
-      <c r="D142" s="43" t="n">
-        <f aca="false">IF(D70=0,0,D140/D70*360)</f>
+      <c r="D24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!D13=0,0,D22/'COMPTE DE RESULTAT'!D13*360)</f>
         <v>141.995353176295</v>
       </c>
-      <c r="E142" s="43" t="n">
-        <f aca="false">IF(E70=0,0,E140/E70*360)</f>
+      <c r="E24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!E13=0,0,E22/'COMPTE DE RESULTAT'!E13*360)</f>
         <v>142.035338771625</v>
       </c>
-      <c r="F142" s="43" t="n">
-        <f aca="false">IF(F70=0,0,F140/F70*360)</f>
+      <c r="F24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!F13=0,0,F22/'COMPTE DE RESULTAT'!F13*360)</f>
         <v>141.657438680371</v>
       </c>
-      <c r="G142" s="43" t="n">
-        <f aca="false">IF(G70=0,0,G140/G70*360)</f>
+      <c r="G24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!G13=0,0,G22/'COMPTE DE RESULTAT'!G13*360)</f>
         <v>141.19462597233</v>
       </c>
-      <c r="H142" s="43" t="n">
-        <f aca="false">IF(H70=0,0,H140/H70*360)</f>
+      <c r="H24" s="45" t="n">
+        <f aca="false">IF('COMPTE DE RESULTAT'!H13=0,0,H22/'COMPTE DE RESULTAT'!H13*360)</f>
         <v>139.911216871306</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="13"/>
-      <c r="B143" s="12" t="s">
-        <v>487</v>
-      </c>
-      <c r="C143" s="44" t="n">
-        <f aca="false">IF(C43=0,0,(C44+C45+C58)/C43)</f>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+      <c r="B25" s="12" t="s">
+        <v>504</v>
+      </c>
+      <c r="C25" s="46" t="n">
+        <f aca="false">IF(BILAN!C43=0,0,(BILAN!C44+BILAN!C45+BILAN!C58)/BILAN!C43)</f>
         <v>0.0587023942433689</v>
       </c>
-      <c r="D143" s="44" t="n">
-        <f aca="false">IF(D43=0,0,(D44+D45+D58)/D43)</f>
+      <c r="D25" s="46" t="n">
+        <f aca="false">IF(BILAN!D43=0,0,(BILAN!D44+BILAN!D45+BILAN!D58)/BILAN!D43)</f>
         <v>0.0214101882884361</v>
       </c>
-      <c r="E143" s="44" t="n">
-        <f aca="false">IF(E43=0,0,(E44+E45+E58)/E43)</f>
-        <v>0</v>
-      </c>
-      <c r="F143" s="44" t="n">
-        <f aca="false">IF(F43=0,0,(F44+F45+F58)/F43)</f>
-        <v>0</v>
-      </c>
-      <c r="G143" s="44" t="n">
-        <f aca="false">IF(G43=0,0,(G44+G45+G58)/G43)</f>
-        <v>0</v>
-      </c>
-      <c r="H143" s="44" t="n">
-        <f aca="false">IF(H43=0,0,(H44+H45+H58)/H43)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="13"/>
-      <c r="B144" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="C144" s="42" t="n">
-        <f aca="false">IF(C43=0,0,C104/C43)</f>
+      <c r="E25" s="46" t="n">
+        <f aca="false">IF(BILAN!E43=0,0,(BILAN!E44+BILAN!E45+BILAN!E58)/BILAN!E43)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="46" t="n">
+        <f aca="false">IF(BILAN!F43=0,0,(BILAN!F44+BILAN!F45+BILAN!F58)/BILAN!F43)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="46" t="n">
+        <f aca="false">IF(BILAN!G43=0,0,(BILAN!G44+BILAN!G45+BILAN!G58)/BILAN!G43)</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="46" t="n">
+        <f aca="false">IF(BILAN!H43=0,0,(BILAN!H44+BILAN!H45+BILAN!H58)/BILAN!H43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13"/>
+      <c r="B26" s="12" t="s">
+        <v>505</v>
+      </c>
+      <c r="C26" s="44" t="n">
+        <f aca="false">IF(BILAN!C43=0,0,'COMPTE DE RESULTAT'!C47/BILAN!C43)</f>
         <v>0.0848791418170092</v>
       </c>
-      <c r="D144" s="42" t="n">
-        <f aca="false">IF(D43=0,0,D104/D43)</f>
+      <c r="D26" s="44" t="n">
+        <f aca="false">IF(BILAN!D43=0,0,'COMPTE DE RESULTAT'!D47/BILAN!D43)</f>
         <v>0.0752224354319878</v>
       </c>
-      <c r="E144" s="42" t="n">
-        <f aca="false">IF(E43=0,0,E104/E43)</f>
+      <c r="E26" s="44" t="n">
+        <f aca="false">IF(BILAN!E43=0,0,'COMPTE DE RESULTAT'!E47/BILAN!E43)</f>
         <v>0.0734776134356451</v>
       </c>
-      <c r="F144" s="42" t="n">
-        <f aca="false">IF(F43=0,0,F104/F43)</f>
+      <c r="F26" s="44" t="n">
+        <f aca="false">IF(BILAN!F43=0,0,'COMPTE DE RESULTAT'!F47/BILAN!F43)</f>
         <v>0.074299771858321</v>
       </c>
-      <c r="G144" s="42" t="n">
-        <f aca="false">IF(G43=0,0,G104/G43)</f>
+      <c r="G26" s="44" t="n">
+        <f aca="false">IF(BILAN!G43=0,0,'COMPTE DE RESULTAT'!G47/BILAN!G43)</f>
         <v>0.0754199169704545</v>
       </c>
-      <c r="H144" s="42" t="n">
-        <f aca="false">IF(H43=0,0,H104/H43)</f>
+      <c r="H26" s="44" t="n">
+        <f aca="false">IF(BILAN!H43=0,0,'COMPTE DE RESULTAT'!H47/BILAN!H43)</f>
         <v>0.080763370731434</v>
-      </c>
-    </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="36" t="s">
-        <v>265</v>
-      </c>
-      <c r="B146" s="36" t="s">
-        <v>489</v>
-      </c>
-      <c r="C146" s="36" t="str">
-        <f aca="false">"Réel "&amp;HYPOTHESES!$C$5</f>
-        <v>Réel 2024</v>
-      </c>
-      <c r="D146" s="37" t="n">
-        <f aca="false">HYPOTHESES!$C$5+1</f>
-        <v>2025</v>
-      </c>
-      <c r="E146" s="37" t="n">
-        <f aca="false">HYPOTHESES!$C$5+2</f>
-        <v>2026</v>
-      </c>
-      <c r="F146" s="37" t="n">
-        <f aca="false">HYPOTHESES!$C$5+3</f>
-        <v>2027</v>
-      </c>
-      <c r="G146" s="37" t="n">
-        <f aca="false">HYPOTHESES!$C$5+4</f>
-        <v>2028</v>
-      </c>
-      <c r="H146" s="37" t="n">
-        <f aca="false">HYPOTHESES!$C$5+5</f>
-        <v>2029</v>
-      </c>
-      <c r="I146" s="36" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="13"/>
-      <c r="B147" s="12" t="s">
-        <v>490</v>
-      </c>
-      <c r="C147" s="15" t="n">
-        <f aca="false">BALANCES!D92</f>
-        <v>0</v>
-      </c>
-      <c r="D147" s="15" t="n">
-        <f aca="false">BALANCES!F92</f>
-        <v>0</v>
-      </c>
-      <c r="E147" s="15" t="n">
-        <f aca="false">BALANCES!H92</f>
-        <v>0</v>
-      </c>
-      <c r="F147" s="15" t="n">
-        <f aca="false">BALANCES!J92</f>
-        <v>0</v>
-      </c>
-      <c r="G147" s="15" t="n">
-        <f aca="false">BALANCES!L92</f>
-        <v>0</v>
-      </c>
-      <c r="H147" s="15" t="n">
-        <f aca="false">BALANCES!N92</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="13"/>
-      <c r="B148" s="12" t="s">
-        <v>491</v>
-      </c>
-      <c r="C148" s="18" t="n">
-        <f aca="false">C30-C60</f>
-        <v>0</v>
-      </c>
-      <c r="D148" s="18" t="n">
-        <f aca="false">D30-D60</f>
-        <v>0</v>
-      </c>
-      <c r="E148" s="18" t="n">
-        <f aca="false">E30-E60</f>
-        <v>0</v>
-      </c>
-      <c r="F148" s="18" t="n">
-        <f aca="false">F30-F60</f>
-        <v>0</v>
-      </c>
-      <c r="G148" s="18" t="n">
-        <f aca="false">G30-G60</f>
-        <v>0</v>
-      </c>
-      <c r="H148" s="18" t="n">
-        <f aca="false">H30-H60</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="13"/>
-      <c r="B149" s="12" t="s">
-        <v>492</v>
-      </c>
-      <c r="C149" s="15" t="n">
-        <f aca="false">C104-HYPOTHESES!C92</f>
-        <v>0</v>
-      </c>
-      <c r="D149" s="15" t="n">
-        <f aca="false">D104-HYPOTHESES!D92</f>
-        <v>0</v>
-      </c>
-      <c r="E149" s="15" t="n">
-        <f aca="false">E104-HYPOTHESES!E92</f>
-        <v>0</v>
-      </c>
-      <c r="F149" s="15" t="n">
-        <f aca="false">F104-HYPOTHESES!F92</f>
-        <v>0</v>
-      </c>
-      <c r="G149" s="15" t="n">
-        <f aca="false">G104-HYPOTHESES!G92</f>
-        <v>0</v>
-      </c>
-      <c r="H149" s="15" t="n">
-        <f aca="false">H104-HYPOTHESES!H92</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="13"/>
-      <c r="B150" s="12" t="s">
-        <v>493</v>
-      </c>
-      <c r="C150" s="41" t="s">
-        <v>428</v>
-      </c>
-      <c r="D150" s="18" t="n">
-        <f aca="false">D131-(D28-D58)</f>
-        <v>0</v>
-      </c>
-      <c r="E150" s="18" t="n">
-        <f aca="false">E131-(E28-E58)</f>
-        <v>0</v>
-      </c>
-      <c r="F150" s="18" t="n">
-        <f aca="false">F131-(F28-F58)</f>
-        <v>0</v>
-      </c>
-      <c r="G150" s="18" t="n">
-        <f aca="false">G131-(G28-G58)</f>
-        <v>0</v>
-      </c>
-      <c r="H150" s="18" t="n">
-        <f aca="false">H131-(H28-H58)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="13"/>
-      <c r="B151" s="12" t="s">
-        <v>494</v>
-      </c>
-      <c r="C151" s="32" t="n">
-        <f aca="false">IF(C28-C58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D151" s="32" t="n">
-        <f aca="false">IF(D28-D58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E151" s="32" t="n">
-        <f aca="false">IF(E28-E58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F151" s="32" t="n">
-        <f aca="false">IF(F28-F58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G151" s="32" t="n">
-        <f aca="false">IF(G28-G58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H151" s="32" t="n">
-        <f aca="false">IF(H28-H58&lt;0,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="13"/>
-      <c r="B152" s="12" t="s">
-        <v>495</v>
-      </c>
-      <c r="C152" s="32" t="n">
-        <f aca="false">IF(C43&lt;C33/2,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D152" s="32" t="n">
-        <f aca="false">IF(D43&lt;D33/2,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E152" s="32" t="n">
-        <f aca="false">IF(E43&lt;E33/2,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F152" s="32" t="n">
-        <f aca="false">IF(F43&lt;F33/2,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G152" s="32" t="n">
-        <f aca="false">IF(G43&lt;G33/2,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H152" s="32" t="n">
-        <f aca="false">IF(H43&lt;H33/2,1,0)</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Approvisionnement caisse = 20 % des sorties de banque via le 585
Soldes de banque et de caisse inchangés ; seul le volume des mouvements
571 / 585 évolue avec le taux saisi dans HYPOTHESES.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017qsfV16W64D6M2WCay1xb5
</commit_message>
<xml_diff>
--- a/previsions/PREVISIONS_FINANCIERES_5ANS_SYSCOHADA.xlsx
+++ b/previsions/PREVISIONS_FINANCIERES_5ANS_SYSCOHADA.xlsx
@@ -189,13 +189,13 @@
     <t xml:space="preserve">   Dette fournisseurs d'investissement au 31/12 (poste DH du bilan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Approvisionnement de la caisse par la banque (virement de fonds 585)</t>
+    <t xml:space="preserve">Part des sorties de banque affectée à l'approvisionnement de la caisse (virement de fonds 585)</t>
   </si>
   <si>
     <t xml:space="preserve">571 / 585</t>
   </si>
   <si>
-    <t xml:space="preserve">Seule entrée en caisse : chèque de retrait banque (D 585 / C 521 puis D 571 / C 585). Créances clients encaissées par chèque ou virement. Défaut : appro réelle 2024.</t>
+    <t xml:space="preserve">Appro caisse = % x mouvements crédit du 521. Seule entrée en caisse (D 585 / C 521 puis D 571 / C 585). Créances clients encaissées par chèque ou virement. Soldes banque et caisse inchangés.</t>
   </si>
   <si>
     <t xml:space="preserve">Ajustement des autres dettes (+ augmentation / - diminution de l'année)</t>
@@ -3084,20 +3084,20 @@
       <c r="B29" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D29" s="16" t="n">
-        <v>6589458</v>
-      </c>
-      <c r="E29" s="16" t="n">
-        <v>6589458</v>
-      </c>
-      <c r="F29" s="16" t="n">
-        <v>6589458</v>
-      </c>
-      <c r="G29" s="16" t="n">
-        <v>6589458</v>
-      </c>
-      <c r="H29" s="16" t="n">
-        <v>6589458</v>
+      <c r="D29" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>0.2</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>54</v>
@@ -13925,12 +13925,12 @@
         <v>0</v>
       </c>
       <c r="F46" s="15" t="n">
-        <f aca="false">HYPOTHESES!D$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!D$29*G45</f>
+        <v>179859044.854246</v>
       </c>
       <c r="G46" s="15" t="n">
-        <f aca="false">HYPOTHESES!D$29+(D46-E46)-(H46-I46)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!D$29*G45+(D46-E46)-(H46-I46)</f>
+        <v>179859044.854246</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46</f>
@@ -13964,12 +13964,12 @@
         <v>0</v>
       </c>
       <c r="F47" s="15" t="n">
-        <f aca="false">HYPOTHESES!D$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!D$29*G45</f>
+        <v>179859044.854246</v>
       </c>
       <c r="G47" s="15" t="n">
-        <f aca="false">HYPOTHESES!D$29+(D47-E47)-(H47-I47)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!D$29*G45+(D47-E47)-(H47-I47)</f>
+        <v>179859044.854246</v>
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47</f>
@@ -15692,11 +15692,11 @@
       </c>
       <c r="F96" s="36" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>3537270852.82874</v>
+        <v>3883810026.53724</v>
       </c>
       <c r="G96" s="36" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>3537270852.82874</v>
+        <v>3883810026.53724</v>
       </c>
       <c r="H96" s="36" t="n">
         <f aca="false">SUM(H5:H94)</f>
@@ -17412,12 +17412,12 @@
         <v>0</v>
       </c>
       <c r="F46" s="15" t="n">
-        <f aca="false">HYPOTHESES!E$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!E$29*G45</f>
+        <v>163602054.930847</v>
       </c>
       <c r="G46" s="15" t="n">
-        <f aca="false">HYPOTHESES!E$29+(D46-E46)-(H46-I46)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!E$29*G45+(D46-E46)-(H46-I46)</f>
+        <v>163602054.930847</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46</f>
@@ -17451,12 +17451,12 @@
         <v>0</v>
       </c>
       <c r="F47" s="15" t="n">
-        <f aca="false">HYPOTHESES!E$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!E$29*G45</f>
+        <v>163602054.930847</v>
       </c>
       <c r="G47" s="15" t="n">
-        <f aca="false">HYPOTHESES!E$29+(D47-E47)-(H47-I47)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!E$29*G45+(D47-E47)-(H47-I47)</f>
+        <v>163602054.930847</v>
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47</f>
@@ -19179,11 +19179,11 @@
       </c>
       <c r="F96" s="36" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>3552342335.84718</v>
+        <v>3866367529.70888</v>
       </c>
       <c r="G96" s="36" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>3552342335.84718</v>
+        <v>3866367529.70888</v>
       </c>
       <c r="H96" s="36" t="n">
         <f aca="false">SUM(H5:H94)</f>
@@ -20899,12 +20899,12 @@
         <v>0</v>
       </c>
       <c r="F46" s="15" t="n">
-        <f aca="false">HYPOTHESES!F$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!F$29*G45</f>
+        <v>161355553.370784</v>
       </c>
       <c r="G46" s="15" t="n">
-        <f aca="false">HYPOTHESES!F$29+(D46-E46)-(H46-I46)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!F$29*G45+(D46-E46)-(H46-I46)</f>
+        <v>161355553.370784</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46</f>
@@ -20938,12 +20938,12 @@
         <v>0</v>
       </c>
       <c r="F47" s="15" t="n">
-        <f aca="false">HYPOTHESES!F$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!F$29*G45</f>
+        <v>161355553.370784</v>
       </c>
       <c r="G47" s="15" t="n">
-        <f aca="false">HYPOTHESES!F$29+(D47-E47)-(H47-I47)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!F$29*G45+(D47-E47)-(H47-I47)</f>
+        <v>161355553.370784</v>
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47</f>
@@ -22666,11 +22666,11 @@
       </c>
       <c r="F96" s="36" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>3681108436.27262</v>
+        <v>3990640627.01418</v>
       </c>
       <c r="G96" s="36" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>3681108436.27262</v>
+        <v>3990640627.01419</v>
       </c>
       <c r="H96" s="36" t="n">
         <f aca="false">SUM(H5:H94)</f>
@@ -24386,12 +24386,12 @@
         <v>0</v>
       </c>
       <c r="F46" s="15" t="n">
-        <f aca="false">HYPOTHESES!G$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!G$29*G45</f>
+        <v>174239968.653212</v>
       </c>
       <c r="G46" s="15" t="n">
-        <f aca="false">HYPOTHESES!G$29+(D46-E46)-(H46-I46)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!G$29*G45+(D46-E46)-(H46-I46)</f>
+        <v>174239968.653212</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46</f>
@@ -24425,12 +24425,12 @@
         <v>0</v>
       </c>
       <c r="F47" s="15" t="n">
-        <f aca="false">HYPOTHESES!G$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!G$29*G45</f>
+        <v>174239968.653212</v>
       </c>
       <c r="G47" s="15" t="n">
-        <f aca="false">HYPOTHESES!G$29+(D47-E47)-(H47-I47)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!G$29*G45+(D47-E47)-(H47-I47)</f>
+        <v>174239968.653212</v>
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47</f>
@@ -26153,11 +26153,11 @@
       </c>
       <c r="F96" s="36" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>3923084886.69319</v>
+        <v>4258385907.99962</v>
       </c>
       <c r="G96" s="36" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>3923084886.69319</v>
+        <v>4258385907.99962</v>
       </c>
       <c r="H96" s="36" t="n">
         <f aca="false">SUM(H5:H94)</f>
@@ -27873,12 +27873,12 @@
         <v>0</v>
       </c>
       <c r="F46" s="15" t="n">
-        <f aca="false">HYPOTHESES!H$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!H$29*G45</f>
+        <v>180492050.539484</v>
       </c>
       <c r="G46" s="15" t="n">
-        <f aca="false">HYPOTHESES!H$29+(D46-E46)-(H46-I46)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!H$29*G45+(D46-E46)-(H46-I46)</f>
+        <v>180492050.539484</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46</f>
@@ -27912,12 +27912,12 @@
         <v>0</v>
       </c>
       <c r="F47" s="15" t="n">
-        <f aca="false">HYPOTHESES!H$29</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!H$29*G45</f>
+        <v>180492050.539484</v>
       </c>
       <c r="G47" s="15" t="n">
-        <f aca="false">HYPOTHESES!H$29+(D47-E47)-(H47-I47)</f>
-        <v>6589458</v>
+        <f aca="false">HYPOTHESES!H$29*G45+(D47-E47)-(H47-I47)</f>
+        <v>180492050.539484</v>
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47</f>
@@ -29640,11 +29640,11 @@
       </c>
       <c r="F96" s="36" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>4065131364.24591</v>
+        <v>4412936549.32488</v>
       </c>
       <c r="G96" s="36" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>4065131364.24591</v>
+        <v>4412936549.32488</v>
       </c>
       <c r="H96" s="36" t="n">
         <f aca="false">SUM(H5:H94)</f>

</xml_diff>